<commit_message>
AI RMF question pilot round 3: prompt fixes, MAP 1.4 and MAP 3.2 decided
- Generator: a row's core keeps its main subject and folded outcomes (split if too
  much); similar single-row questions must still share; producer's own model, data and
  build are framed by the model, not "highest-criticality AI systems".
- Evaluator: a flagged base-model question is not a duplicate of a general third-party
  question; compares every pair of single-row questions; trimming may not drop the row's
  main subject.
- criticality_frame_optional adds model_building, model, test_tuning_data.
- Decided in the review sheet: MAP 1.4 Q3 (business purpose only), MAP 3.2 internal
  process split in two (cost of wrong output; likelihood and size, folded MAP 5.1).
- Round 3 recorded: GOVERN 6.1 (pass, base-model question back), MEASURE 2.7 (needs
  human review: Q4 near-duplicate of Q2).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ai/authoring/questions_areas.xlsx
+++ b/data/ai/authoring/questions_areas.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Read me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Area questions'!$A$1:$M$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Area questions'!$A$1:$M$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -568,7 +568,7 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>For the AI features inside vendor products you use, how do you decide what business purpose they serve and which of your data they may work on? Who owns that decision?</t>
+          <t>For the AI features inside vendor products you use, how do you decide what business purpose they serve? Who owns that decision?</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -672,17 +672,13 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Chains two things to answer (business purpose and which data they may work on); the data part is not supported by the cited action about business value.</t>
-        </is>
-      </c>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
@@ -725,23 +721,19 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>MAP 3.2 — suggested action 6, MAP 5.1 — suggested action 3</t>
+          <t>MAP 3.2 — suggested action 6</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>Row is shared with folded MAP 5.1 (likelihood and magnitude, benefits as well as costs, identifying high-impact decisions) but the question asks only for the cost of wrong output.</t>
-        </is>
-      </c>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
@@ -763,12 +755,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>customer_facing</t>
+          <t>internal_process</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Customer-facing application</t>
+          <t>Internal process</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -779,12 +771,12 @@
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how are the costs to customers and to the business of wrong, harmful or leaked answers reaching customers examined and documented? Who reviews this?</t>
+          <t>For your highest-criticality AI systems, how do you rate how likely and how large the effects of AI in internal decisions are, benefits as well as harms? Who reviews these ratings?</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>MAP 3.2 — suggested action 6</t>
+          <t>MAP 5.1 — suggested action 3</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
@@ -796,7 +788,7 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
@@ -818,12 +810,12 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>output</t>
+          <t>customer_facing</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Output</t>
+          <t>Customer-facing application</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -834,12 +826,12 @@
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how do you work out the cost of wrong, manipulated or biased AI answers and who could be harmed by acting on them? Where is this recorded?</t>
+          <t>For your highest-criticality AI systems, how are the costs to customers and to the business of wrong, harmful or leaked answers reaching customers examined and documented? Who reviews this?</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>MAP 3.2 — suggested action 1</t>
+          <t>MAP 3.2 — suggested action 6</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
@@ -851,7 +843,7 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
@@ -873,12 +865,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>hosting</t>
+          <t>output</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Output</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -889,12 +881,12 @@
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how are the costs of a hosting compromise, outage or cost abuse (stolen compute, runaway spend, downtime) examined and compared with your risk tolerance? Who owns this?</t>
+          <t>For your highest-criticality AI systems, how do you work out the cost of wrong, manipulated or biased AI answers and who could be harmed by acting on them? Where is this recorded?</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>MAP 3.2 — suggested action 6</t>
+          <t>MAP 3.2 — suggested action 1</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
@@ -906,34 +898,34 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8</t>
+          <t>MAP 3.2</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+          <t>Potential costs, including non-monetary costs, which result from expected or realized AI errors or system functionality and trustworthiness - as connected to organizational risk tolerance - are examined and documented.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>internal_process, customer_facing</t>
+          <t>hosting</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Internal process; Customer-facing application</t>
+          <t>Hosting</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -944,19 +936,15 @@
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how is the AI's part in each decision or customer answer recorded, including human review, overrides and the output that was relied on, so that a high-impact decision or answer can be audited later? Who reviews these records, and how long are they kept?</t>
+          <t>For your highest-criticality AI systems, how are the costs of a hosting compromise, outage or cost abuse (stolen compute, runaway spend, downtime) examined and compared with your risk tolerance? Who owns this?</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8 — suggested action 1, MEASURE 2.8 — suggested action 6</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>LLM-8.1, LLM-8.2, LLM-8.5, LLM-8.10</t>
-        </is>
-      </c>
+          <t>MAP 3.2 — suggested action 6</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -972,17 +960,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8</t>
+          <t>MEASURE 2.7</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+          <t>AI system security and resilience – as identified in the MAP function – are evaluated and documented.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1003,17 +991,17 @@
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>For AI code generation, how is its use logged, including who used which tool, what was generated and what was merged, so that AI-written code and the prompts behind it can be traced? Who can look at these records?</t>
+          <t>How is your AI coding assistant tested for AI-specific weaknesses, for example suggesting invented or malicious packages? Where are the results recorded?</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8 — suggested action 1</t>
+          <t>MEASURE 2.7 — suggested action 2</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.1, LLM-8.2, LLM-8.5</t>
+          <t>LLM-16.3</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1024,34 +1012,34 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>agent</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8</t>
+          <t>MEASURE 2.7</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+          <t>AI system security and resilience – as identified in the MAP function – are evaluated and documented.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>vendor_ai</t>
+          <t>customer_facing</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Vendor AI</t>
+          <t>Customer-facing application</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1062,17 +1050,17 @@
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>For the AI features your vendors run on your data, how can you trace what the AI did with your data, through the vendor's own logs or your own? How often does someone review that activity, and what evidence of the review exists?</t>
+          <t>For your highest-criticality AI systems facing the public, how is abuse by public users tested, for example prompt injection? How are results documented and acted on?</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8 — suggested action 1</t>
+          <t>MEASURE 2.7 — suggested action 2, MEASURE 2.7 — suggested action 3</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.12, LLM-8.2, LLM-8.1</t>
+          <t>LLM-18.2, LLM-16.13</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1083,55 +1071,55 @@
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>agent</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8</t>
+          <t>MEASURE 2.7</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+          <t>AI system security and resilience – as identified in the MAP function – are evaluated and documented.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>model_building</t>
+          <t>invisible_usage</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Model building</t>
+          <t>Invisible AI usage (unapproved or external)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>producer</t>
+          <t>none, consumer, producer</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>For the model you build or tune, how are build, tuning and release events logged, showing who did what and when, so that changes to the model and its releases can be traced and accounted for? Who reviews these records?</t>
+          <t>How do you test and measure how your systems hold up to other people's AI agents, scrapers and MCP clients acting at machine speed, for example through authentication and throttling? Where are the results recorded?</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8 — suggested action 1</t>
+          <t>MEASURE 2.7 — suggested action 1, MEASURE 2.7 — suggested action 5</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.1, LLM-8.2</t>
+          <t>LLM-13.3, MCP-13.10, AGENT-13.10</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1142,114 +1130,118 @@
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>agent</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8</t>
+          <t>MEASURE 2.7</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+          <t>AI system security and resilience – as identified in the MAP function – are evaluated and documented.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>invisible_usage</t>
+          <t>output</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Invisible AI usage (unapproved or external)</t>
+          <t>Output</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>none, consumer, producer</t>
+          <t>consumer, producer</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>How do your logs show AI use you did not choose — AI services your staff reach, and outside AI agents or tools calling your systems — and under whose identity? Who reviews this?</t>
+          <t>For your highest-criticality AI systems, how are the AI's answers tested against attacker steering, for example prompt injection through user input or retrieved content? Where are the results documented?</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8 — suggested action 1</t>
+          <t>MEASURE 2.7 — suggested action 2, MEASURE 2.7 — suggested action 3</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.1, LLM-8.2, LLM-8.6, MCP-8.2</t>
+          <t>LLM-16.3, LLM-18.2</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>pass</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr"/>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Tests AI answers against prompt injection, the same practice (and same cis_refs LLM-18.2) as question 2 on customer_facing; the public-user abuse test already covers steering of answers, so the two split one practice.</t>
+        </is>
+      </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>agent</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8</t>
+          <t>MEASURE 2.7</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+          <t>AI system security and resilience – as identified in the MAP function – are evaluated and documented.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>input</t>
+          <t>test_tuning_data</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Test, tuning and evaluation data</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>consumer, producer</t>
+          <t>producer</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how are prompts and responses logged as a record of who sent what? Who can read those logs, and how long are they kept?</t>
+          <t>For the models behind your most critical AI systems, how are training, tuning and evaluation data and the test harness checked and protected against poisoning and tampering, for example changes that hide failures? Who reviews changes to them?</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8 — suggested action 1</t>
+          <t>MEASURE 2.7 — suggested action 2</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.1, LLM-8.2, LLM-8.5, LLM-8.3</t>
+          <t>LLM-3.1, LLM-3.3, LLM-6.8</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1260,57 +1252,53 @@
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>agent</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8</t>
+          <t>MEASURE 2.7</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+          <t>AI system security and resilience – as identified in the MAP function – are evaluated and documented.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>output</t>
+          <t>model</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Output</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>consumer, producer</t>
+          <t>producer</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, when an answer turns out to be wrong or manipulated, how do your records let you trace how it came about — which model version, instructions and sources produced it — and who or what relied on it? Who owns this?</t>
+          <t>For the models behind your most critical AI systems, how is the model tested against theft, extraction through the API and tampering with versions? Where are the results documented?</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8 — suggested action 1</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>LLM-8.2, LLM-8.5</t>
-        </is>
-      </c>
+          <t>MEASURE 2.7 — suggested action 3, MEASURE 2.7 — suggested action 10</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1319,55 +1307,55 @@
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>agent</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8</t>
+          <t>MEASURE 2.7</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+          <t>AI system security and resilience – as identified in the MAP function – are evaluated and documented.</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>test_tuning_data</t>
+          <t>source_data</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Test, tuning and evaluation data</t>
+          <t>Source data (RAG / knowledge graph)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>producer</t>
+          <t>consumer, producer</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>For the training, tuning and evaluation data and the test harness you use, how are changes and access logged and tied to a named person, so that tampering or misuse can be traced? Who reviews these records?</t>
+          <t>For your highest-criticality AI systems, how is the AI's retrieval from your data stores tested, for example that users only see what they are entitled to and that content cannot be poisoned or copied out? Where are the results recorded?</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8 — suggested action 1</t>
+          <t>MEASURE 2.7 — suggested action 2</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.2, LLM-8.1</t>
+          <t>LLM-3.3, LLM-3.12</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1378,55 +1366,55 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>agent</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8</t>
+          <t>MEASURE 2.7</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+          <t>AI system security and resilience – as identified in the MAP function – are evaluated and documented.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>mcp_tools</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>MCP / tools (inside or outside)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>producer</t>
+          <t>consumer, producer</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>For your own model, how are access to its weights, system prompts and configurations, and changes to model versions, logged so that copying or tampering can be traced to a person? Who reviews these records and how long are they kept?</t>
+          <t>For your highest-criticality AI systems, how are the tools and MCP servers the AI can call tested for security, for example prompt injection driving tool calls or a changed server? Where are the results recorded?</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8 — suggested action 1</t>
+          <t>MEASURE 2.7 — suggested action 2, MEASURE 2.7 — suggested action 3</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.1, LLM-8.2, LLM-8.10</t>
+          <t>MCP-16.13</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1437,34 +1425,34 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>agent</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8</t>
+          <t>MEASURE 2.7</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+          <t>AI system security and resilience – as identified in the MAP function – are evaluated and documented.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>source_data</t>
+          <t>agent</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Source data (RAG / knowledge graph)</t>
+          <t>Agent</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1475,17 +1463,17 @@
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>For the data your AI retrieves to answer questions, how are retrievals and changes to that data logged, showing who asked and what was returned, so that access to sensitive content through the AI can be traced? Who reviews these logs?</t>
+          <t>For your highest-criticality AI agents, how is security tested with adversarial or red-team exercises, for example manipulated input that triggers actions? How are the results documented and acted on?</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8 — suggested action 1</t>
+          <t>MEASURE 2.7 — suggested action 2, MEASURE 2.7 — suggested action 3</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.2, LLM-3.14</t>
+          <t>AGENT-16.13, AGENT-18.1, AGENT-18.5, AGENT-18.2</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1496,34 +1484,34 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>agent</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8</t>
+          <t>MEASURE 2.7</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+          <t>AI system security and resilience – as identified in the MAP function – are evaluated and documented.</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>mcp_tools, agent</t>
+          <t>hosting</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>MCP / tools (inside or outside); Agent</t>
+          <t>Hosting</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1534,17 +1522,17 @@
       <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how is each action the AI takes through tools or on your systems logged, with the credentials or identity it used and what it did, so that it can be traced back to the request and approval behind it? Who reviews these logs, and how long are they kept?</t>
+          <t>For your highest-criticality AI systems that you host, how are the hosting environment and exposed AI endpoints tested for security and resilience, for example through vulnerability scans? Who follows up on the findings?</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8 — suggested action 1</t>
+          <t>MEASURE 2.7 — suggested action 1, MEASURE 2.7 — suggested action 2</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>MCP-8.1, MCP-8.2, MCP-8.5, AGENT-8.1, AGENT-8.2, AGENT-8.5, AGENT-8.9</t>
+          <t>LLM-7.5, LLM-7.6, LLM-13.3</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1555,7 +1543,7 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>agent</t>
         </is>
       </c>
     </row>
@@ -1572,17 +1560,17 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>hosting</t>
+          <t>internal_process, customer_facing</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Internal process; Customer-facing application</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1593,17 +1581,17 @@
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>For the environment where you host AI models, how are administrative actions, model registry changes, secret access and serving endpoint activity logged so that actions can be traced and accounted for? Who reviews them, and how often?</t>
+          <t>For your highest-criticality AI systems, how is the AI's part in each decision or customer answer recorded, including human review, overrides and the output that was relied on, so that a high-impact decision or answer can be audited later? Who reviews these records, and how long are they kept?</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8 — suggested action 1</t>
+          <t>MEASURE 2.8 — suggested action 1, MEASURE 2.8 — suggested action 6</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.2, LLM-8.1, LLM-8.9</t>
+          <t>LLM-8.1, LLM-8.2, LLM-8.5, LLM-8.10</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1621,52 +1609,48 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>MANAGE 3.2</t>
+          <t>MEASURE 2.8</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Pre-trained models which are used for development are monitored as part of AI system regular monitoring and maintenance.</t>
+          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>model_building</t>
+          <t>code_generation</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Model building</t>
+          <t>Code generation</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>producer</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>built_on_existing_model</t>
-        </is>
-      </c>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>For the pre-trained base models you build on, how are they tracked and monitored, for example for published vulnerabilities? Who owns this?</t>
+          <t>For AI code generation, how is its use logged, including who used which tool, what was generated and what was merged, so that AI-written code and the prompts behind it can be traced? Who can look at these records?</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>MANAGE 3.2 — suggested action 1, MANAGE 3.2 — suggested action 2</t>
+          <t>MEASURE 2.8 — suggested action 1</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>LLM-16.2, LLM-2.1</t>
+          <t>LLM-8.1, LLM-8.2, LLM-8.5</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1677,14 +1661,667 @@
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr">
         <is>
+          <t>human</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>vendor_ai</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Vendor AI</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>For the AI features your vendors run on your data, how can you trace what the AI did with your data, through the vendor's own logs or your own? How often does someone review that activity, and what evidence of the review exists?</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>LLM-8.12, LLM-8.2, LLM-8.1</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>model_building</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Model building</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>producer</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>For the model you build or tune, how are build, tuning and release events logged, showing who did what and when, so that changes to the model and its releases can be traced and accounted for? Who reviews these records?</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>LLM-8.1, LLM-8.2</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>invisible_usage</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Invisible AI usage (unapproved or external)</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>none, consumer, producer</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>How do your logs show AI use you did not choose — AI services your staff reach, and outside AI agents or tools calling your systems — and under whose identity? Who reviews this?</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>LLM-8.1, LLM-8.2, LLM-8.6, MCP-8.2</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>For your highest-criticality AI systems, how are prompts and responses logged as a record of who sent what? Who can read those logs, and how long are they kept?</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>LLM-8.1, LLM-8.2, LLM-8.5, LLM-8.3</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>For your highest-criticality AI systems, when an answer turns out to be wrong or manipulated, how do your records let you trace how it came about — which model version, instructions and sources produced it — and who or what relied on it? Who owns this?</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>LLM-8.2, LLM-8.5</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>test_tuning_data</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Test, tuning and evaluation data</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>producer</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>For the training, tuning and evaluation data and the test harness you use, how are changes and access logged and tied to a named person, so that tampering or misuse can be traced? Who reviews these records?</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>LLM-8.2, LLM-8.1</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>producer</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>For your own model, how are access to its weights, system prompts and configurations, and changes to model versions, logged so that copying or tampering can be traced to a person? Who reviews these records and how long are they kept?</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>LLM-8.1, LLM-8.2, LLM-8.10</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>source_data</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Source data (RAG / knowledge graph)</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>For the data your AI retrieves to answer questions, how are retrievals and changes to that data logged, showing who asked and what was returned, so that access to sensitive content through the AI can be traced? Who reviews these logs?</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>LLM-8.2, LLM-3.14</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>mcp_tools, agent</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>MCP / tools (inside or outside); Agent</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>For your highest-criticality AI systems, how is each action the AI takes through tools or on your systems logged, with the credentials or identity it used and what it did, so that it can be traced back to the request and approval behind it? Who reviews these logs, and how long are they kept?</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>MCP-8.1, MCP-8.2, MCP-8.5, AGENT-8.1, AGENT-8.2, AGENT-8.5, AGENT-8.9</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>hosting</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Hosting</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>For the environment where you host AI models, how are administrative actions, model registry changes, secret access and serving endpoint activity logged so that actions can be traced and accounted for? Who reviews them, and how often?</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 2.8 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>LLM-8.2, LLM-8.1, LLM-8.9</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 3.2</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Pre-trained models which are used for development are monitored as part of AI system regular monitoring and maintenance.</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>model_building</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Model building</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>producer</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>built_on_existing_model</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>For the pre-trained base models you build on, how are they tracked and monitored, for example for published vulnerabilities? Who owns this?</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 3.2 — suggested action 1, MANAGE 3.2 — suggested action 2</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>LLM-16.2, LLM-2.1</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
           <t>agent</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M21"/>
+  <autoFilter ref="A1:M32"/>
   <dataValidations count="1">
-    <dataValidation sqref="K2:K221" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K2:K232" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"pass,needs_human_review"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
AI RMF review decisions of 2026-10-29 (on dd1830c)
- Criticality frame optional for invisible_usage: unapproved AI and outside agents are not
  in the AI system inventory, so they have no criticality to frame by.
- MAP 1.4: internal_process and customer_facing share one question naming no area;
  vendor_ai stays separate.
- MEASURE 2.8 Q10 (source_data) and Q12 (hosting) carry the criticality frame.
- MEASURE 2.7 Q5 cites suggested action 2 (red-team testing) instead of 10 (watermarking).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ai/authoring/questions_areas.xlsx
+++ b/data/ai/authoring/questions_areas.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Read me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Area questions'!$A$1:$M$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Area questions'!$A$1:$M$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -535,12 +535,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>internal_process</t>
+          <t>internal_process, customer_facing</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Internal process</t>
+          <t>Internal process; Customer-facing application</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -551,7 +551,7 @@
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how is the business value of using AI output in each internal workflow defined? Who owns that definition?</t>
+          <t>For your highest-criticality AI systems, how is the business value of the AI's results defined, and who owns that definition?</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -590,12 +590,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>customer_facing</t>
+          <t>vendor_ai</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Customer-facing application</t>
+          <t>Vendor AI</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -606,7 +606,7 @@
       <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how is the business value of your customer-facing AI defined? Who owns that definition?</t>
+          <t>For the AI features inside vendor products you use, how do you decide what business purpose they serve? Who owns that decision?</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -630,27 +630,27 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MAP 1.4</t>
+          <t>MAP 3.2</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>The business value or context of business use has been clearly defined or – in the case of assessing existing AI systems – re-evaluated.</t>
+          <t>Potential costs, including non-monetary costs, which result from expected or realized AI errors or system functionality and trustworthiness - as connected to organizational risk tolerance - are examined and documented.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>vendor_ai</t>
+          <t>internal_process</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Vendor AI</t>
+          <t>Internal process</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -661,12 +661,12 @@
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>For the AI features inside vendor products you use, how do you decide what business purpose they serve? Who owns that decision?</t>
+          <t>For your highest-criticality AI systems, how do you estimate the cost of wrong AI output in internal decisions, for example from past use and feedback? Where is this recorded?</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>MAP 1.4 — suggested action 1</t>
+          <t>MAP 3.2 — suggested action 6</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -716,12 +716,12 @@
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how do you estimate the cost of wrong AI output in internal decisions, for example from past use and feedback? Where is this recorded?</t>
+          <t>For your highest-criticality AI systems, how do you rate how likely and how large the effects of AI in internal decisions are, benefits as well as harms? Who reviews these ratings?</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>MAP 3.2 — suggested action 6</t>
+          <t>MAP 5.1 — suggested action 3</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
@@ -750,17 +750,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>internal_process</t>
+          <t>customer_facing</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Internal process</t>
+          <t>Customer-facing application</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -771,12 +771,12 @@
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how do you rate how likely and how large the effects of AI in internal decisions are, benefits as well as harms? Who reviews these ratings?</t>
+          <t>For your highest-criticality AI systems, how are the costs to customers and to the business of wrong, harmful or leaked answers reaching customers examined and documented? Who reviews this?</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>MAP 5.1 — suggested action 3</t>
+          <t>MAP 3.2 — suggested action 6</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
@@ -805,17 +805,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>customer_facing</t>
+          <t>output</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Customer-facing application</t>
+          <t>Output</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -826,12 +826,12 @@
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how are the costs to customers and to the business of wrong, harmful or leaked answers reaching customers examined and documented? Who reviews this?</t>
+          <t>For your highest-criticality AI systems, how do you work out the cost of wrong, manipulated or biased AI answers and who could be harmed by acting on them? Where is this recorded?</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>MAP 3.2 — suggested action 6</t>
+          <t>MAP 3.2 — suggested action 1</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
@@ -860,17 +860,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>output</t>
+          <t>hosting</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Output</t>
+          <t>Hosting</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -881,12 +881,12 @@
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how do you work out the cost of wrong, manipulated or biased AI answers and who could be harmed by acting on them? Where is this recorded?</t>
+          <t>For your highest-criticality AI systems, how are the costs of a hosting compromise, outage or cost abuse (stolen compute, runaway spend, downtime) examined and compared with your risk tolerance? Who owns this?</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>MAP 3.2 — suggested action 1</t>
+          <t>MAP 3.2 — suggested action 6</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
@@ -905,27 +905,27 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>MAP 3.2</t>
+          <t>MEASURE 2.7</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Potential costs, including non-monetary costs, which result from expected or realized AI errors or system functionality and trustworthiness - as connected to organizational risk tolerance - are examined and documented.</t>
+          <t>AI system security and resilience – as identified in the MAP function – are evaluated and documented.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>hosting</t>
+          <t>code_generation</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Code generation</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -936,15 +936,19 @@
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how are the costs of a hosting compromise, outage or cost abuse (stolen compute, runaway spend, downtime) examined and compared with your risk tolerance? Who owns this?</t>
+          <t>How is the AI coding assistant tested for AI-specific weaknesses, for example suggesting packages that do not exist or are malicious, or being steered by poisoned context? Where are the results recorded?</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>MAP 3.2 — suggested action 6</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr"/>
+          <t>MEASURE 2.7 — suggested action 2</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>LLM-16.3</t>
+        </is>
+      </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -970,17 +974,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>code_generation</t>
+          <t>customer_facing, output</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Code generation</t>
+          <t>Customer-facing application; Output</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -991,17 +995,17 @@
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>How is the AI coding assistant tested for AI-specific weaknesses, for example suggesting packages that do not exist or are malicious, or being steered by poisoned context? Where are the results recorded?</t>
+          <t>For your highest-criticality AI systems, how are the answers tested against prompt injection and other attempts to steer the AI, for example through user input or retrieved content? Where are the results recorded?</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.7 — suggested action 2</t>
+          <t>MEASURE 2.7 — suggested action 2, MEASURE 2.7 — suggested action 3</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>LLM-16.3</t>
+          <t>LLM-18.2, LLM-16.13, LLM-16.3</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1012,7 +1016,7 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
@@ -1029,38 +1033,38 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>customer_facing, output</t>
+          <t>invisible_usage</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Customer-facing application; Output</t>
+          <t>Invisible AI usage (unapproved or external)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>consumer, producer</t>
+          <t>none, consumer, producer</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how are the answers tested against prompt injection and other attempts to steer the AI, for example through user input or retrieved content? Where are the results recorded?</t>
+          <t>How do you test how your systems hold up when other people's AI agents, scrapers or MCP clients act on users' behalf at machine speed, for example through sign-in checks, rate limits or filtering? How often is this tested?</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.7 — suggested action 2, MEASURE 2.7 — suggested action 3</t>
+          <t>MEASURE 2.7 — suggested action 5</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>LLM-18.2, LLM-16.13, LLM-16.3</t>
+          <t>LLM-13.3, MCP-13.10, AGENT-13.10</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1071,7 +1075,7 @@
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
@@ -1088,38 +1092,38 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>invisible_usage</t>
+          <t>test_tuning_data</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Invisible AI usage (unapproved or external)</t>
+          <t>Test, tuning and evaluation data</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>none, consumer, producer</t>
+          <t>producer</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>How do you test how your systems hold up when other people's AI agents, scrapers or MCP clients act on users' behalf at machine speed, for example through sign-in checks, rate limits or filtering? How often is this tested?</t>
+          <t>For the models behind your most critical AI systems, how are the data sets used to build and evaluate the model protected against poisoning and tampering, for example changes made to hide failures? Who reviews changes to them?</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.7 — suggested action 5</t>
+          <t>MEASURE 2.7 — suggested action 2</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>LLM-13.3, MCP-13.10, AGENT-13.10</t>
+          <t>LLM-3.1, LLM-3.3, LLM-6.8</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1130,7 +1134,7 @@
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
@@ -1147,17 +1151,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>test_tuning_data</t>
+          <t>model</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Test, tuning and evaluation data</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1168,7 +1172,7 @@
       <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>For the models behind your most critical AI systems, how are the data sets used to build and evaluate the model protected against poisoning and tampering, for example changes made to hide failures? Who reviews changes to them?</t>
+          <t>For the models behind your most critical AI systems, how is the model tested against theft, extraction through the API and tampering with versions? Where are the results documented?</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1176,11 +1180,7 @@
           <t>MEASURE 2.7 — suggested action 2</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>LLM-3.1, LLM-3.3, LLM-6.8</t>
-        </is>
-      </c>
+      <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1189,7 +1189,7 @@
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
@@ -1206,36 +1206,40 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>source_data</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Source data (RAG / knowledge graph)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>producer</t>
+          <t>consumer, producer</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>For the models behind your most critical AI systems, how is the model tested against theft, extraction through the API and tampering with versions? Where are the results documented?</t>
+          <t>For your highest-criticality AI systems, how is the data the AI retrieves tested so that users only see what they are entitled to, for example by trying to pull out content they should not reach? Where are the results recorded?</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.7 — suggested action 10</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr"/>
+          <t>MEASURE 2.7 — suggested action 2</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>LLM-3.3, LLM-3.12</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1244,7 +1248,7 @@
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
@@ -1261,17 +1265,17 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>source_data</t>
+          <t>mcp_tools</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Source data (RAG / knowledge graph)</t>
+          <t>MCP / tools (inside or outside)</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1282,7 +1286,7 @@
       <c r="G15" s="2" t="inlineStr"/>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how is the data the AI retrieves tested so that users only see what they are entitled to, for example by trying to pull out content they should not reach? Where are the results recorded?</t>
+          <t>For your highest-criticality AI systems, how are the tools and MCP servers the AI can call tested for security, for example prompt injection driving tool calls or permission abuse? Where are the results recorded?</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1292,7 +1296,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>LLM-3.3, LLM-3.12</t>
+          <t>MCP-16.13</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1303,7 +1307,7 @@
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
@@ -1320,17 +1324,17 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>mcp_tools</t>
+          <t>agent</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>MCP / tools (inside or outside)</t>
+          <t>Agent</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1341,17 +1345,17 @@
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how are the tools and MCP servers the AI can call tested for security, for example prompt injection driving tool calls or permission abuse? Where are the results recorded?</t>
+          <t>For your highest-criticality AI systems, how are your AI agents red-teamed, for example with manipulated input that triggers actions? Where are the results documented?</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.7 — suggested action 2</t>
+          <t>MEASURE 2.7 — suggested action 2, MEASURE 2.7 — suggested action 3</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>MCP-16.13</t>
+          <t>AGENT-16.13, AGENT-18.1, AGENT-18.5</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1362,7 +1366,7 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
@@ -1379,17 +1383,17 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>hosting</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Agent</t>
+          <t>Hosting</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1400,17 +1404,17 @@
       <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how are your AI agents red-teamed, for example with manipulated input that triggers actions? Where are the results documented?</t>
+          <t>For your highest-criticality AI systems, how are the servers and exposed endpoints where you host a model tested for security and resilience, for example through vulnerability scans or adversarial exercises? Who acts on the findings?</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.7 — suggested action 2, MEASURE 2.7 — suggested action 3</t>
+          <t>MEASURE 2.7 — suggested action 2</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>AGENT-16.13, AGENT-18.1, AGENT-18.5</t>
+          <t>LLM-7.5, LLM-7.6</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1421,34 +1425,34 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.7</t>
+          <t>MEASURE 2.8</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>AI system security and resilience – as identified in the MAP function – are evaluated and documented.</t>
+          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>hosting</t>
+          <t>internal_process, customer_facing</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Internal process; Customer-facing application</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1459,17 +1463,17 @@
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how are the servers and exposed endpoints where you host a model tested for security and resilience, for example through vulnerability scans or adversarial exercises? Who acts on the findings?</t>
+          <t>For your highest-criticality AI systems, how is the AI's part in each decision or customer answer recorded, including human review, overrides and the output that was relied on, so that a high-impact decision or answer can be audited later? Who reviews these records, and how long are they kept?</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.7 — suggested action 2</t>
+          <t>MEASURE 2.8 — suggested action 1, MEASURE 2.8 — suggested action 6</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>LLM-7.5, LLM-7.6</t>
+          <t>LLM-8.1, LLM-8.2, LLM-8.5, LLM-8.10</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1480,7 +1484,7 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>human</t>
         </is>
       </c>
     </row>
@@ -1497,17 +1501,17 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>internal_process, customer_facing</t>
+          <t>code_generation</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Internal process; Customer-facing application</t>
+          <t>Code generation</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1518,17 +1522,17 @@
       <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how is the AI's part in each decision or customer answer recorded, including human review, overrides and the output that was relied on, so that a high-impact decision or answer can be audited later? Who reviews these records, and how long are they kept?</t>
+          <t>For AI code generation, how is its use logged, including who used which tool, what was generated and what was merged, so that AI-written code and the prompts behind it can be traced? Who can look at these records?</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8 — suggested action 1, MEASURE 2.8 — suggested action 6</t>
+          <t>MEASURE 2.8 — suggested action 1</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.1, LLM-8.2, LLM-8.5, LLM-8.10</t>
+          <t>LLM-8.1, LLM-8.2, LLM-8.5</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1556,17 +1560,17 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>code_generation</t>
+          <t>vendor_ai</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Code generation</t>
+          <t>Vendor AI</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1577,7 +1581,7 @@
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>For AI code generation, how is its use logged, including who used which tool, what was generated and what was merged, so that AI-written code and the prompts behind it can be traced? Who can look at these records?</t>
+          <t>For the AI features your vendors run on your data, how can you trace what the AI did with your data, through the vendor's own logs or your own? How often does someone review that activity, and what evidence of the review exists?</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1587,7 +1591,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.1, LLM-8.2, LLM-8.5</t>
+          <t>LLM-8.12, LLM-8.2, LLM-8.1</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1615,28 +1619,28 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>vendor_ai</t>
+          <t>model_building</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Vendor AI</t>
+          <t>Model building</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>consumer, producer</t>
+          <t>producer</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>For the AI features your vendors run on your data, how can you trace what the AI did with your data, through the vendor's own logs or your own? How often does someone review that activity, and what evidence of the review exists?</t>
+          <t>For the model you build or tune, how are build, tuning and release events logged, showing who did what and when, so that changes to the model and its releases can be traced and accounted for? Who reviews these records?</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1646,7 +1650,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.12, LLM-8.2, LLM-8.1</t>
+          <t>LLM-8.1, LLM-8.2</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1674,28 +1678,28 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>model_building</t>
+          <t>invisible_usage</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Model building</t>
+          <t>Invisible AI usage (unapproved or external)</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>producer</t>
+          <t>none, consumer, producer</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>For the model you build or tune, how are build, tuning and release events logged, showing who did what and when, so that changes to the model and its releases can be traced and accounted for? Who reviews these records?</t>
+          <t>How do your logs show AI use you did not choose — AI services your staff reach, and outside AI agents or tools calling your systems — and under whose identity? Who reviews this?</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1705,7 +1709,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.1, LLM-8.2</t>
+          <t>LLM-8.1, LLM-8.2, LLM-8.6, MCP-8.2</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1733,28 +1737,28 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>invisible_usage</t>
+          <t>input</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Invisible AI usage (unapproved or external)</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>none, consumer, producer</t>
+          <t>consumer, producer</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>How do your logs show AI use you did not choose — AI services your staff reach, and outside AI agents or tools calling your systems — and under whose identity? Who reviews this?</t>
+          <t>For your highest-criticality AI systems, how are prompts and responses logged as a record of who sent what? Who can read those logs, and how long are they kept?</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1764,7 +1768,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.1, LLM-8.2, LLM-8.6, MCP-8.2</t>
+          <t>LLM-8.1, LLM-8.2, LLM-8.5, LLM-8.3</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -1792,17 +1796,17 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>input</t>
+          <t>output</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Output</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1813,7 +1817,7 @@
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how are prompts and responses logged as a record of who sent what? Who can read those logs, and how long are they kept?</t>
+          <t>For your highest-criticality AI systems, when an answer turns out to be wrong or manipulated, how do your records let you trace how it came about — which model version, instructions and sources produced it — and who or what relied on it? Who owns this?</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1823,7 +1827,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.1, LLM-8.2, LLM-8.5, LLM-8.3</t>
+          <t>LLM-8.2, LLM-8.5</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -1851,28 +1855,28 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>output</t>
+          <t>test_tuning_data</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Output</t>
+          <t>Test, tuning and evaluation data</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>consumer, producer</t>
+          <t>producer</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, when an answer turns out to be wrong or manipulated, how do your records let you trace how it came about — which model version, instructions and sources produced it — and who or what relied on it? Who owns this?</t>
+          <t>For the training, tuning and evaluation data and the test harness you use, how are changes and access logged and tied to a named person, so that tampering or misuse can be traced? Who reviews these records?</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1882,7 +1886,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.2, LLM-8.5</t>
+          <t>LLM-8.2, LLM-8.1</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -1910,17 +1914,17 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>test_tuning_data</t>
+          <t>model</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Test, tuning and evaluation data</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1931,7 +1935,7 @@
       <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>For the training, tuning and evaluation data and the test harness you use, how are changes and access logged and tied to a named person, so that tampering or misuse can be traced? Who reviews these records?</t>
+          <t>For your own model, how are access to its weights, system prompts and configurations, and changes to model versions, logged so that copying or tampering can be traced to a person? Who reviews these records and how long are they kept?</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1941,7 +1945,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.2, LLM-8.1</t>
+          <t>LLM-8.1, LLM-8.2, LLM-8.10</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -1969,28 +1973,28 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>source_data</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Source data (RAG / knowledge graph)</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>producer</t>
+          <t>consumer, producer</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>For your own model, how are access to its weights, system prompts and configurations, and changes to model versions, logged so that copying or tampering can be traced to a person? Who reviews these records and how long are they kept?</t>
+          <t>For your highest-criticality AI systems, how are retrievals from the data your AI looks up, and changes to that data, logged, showing who asked and what was returned, so that access to sensitive content through the AI can be traced? Who reviews these logs?</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -2000,7 +2004,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.1, LLM-8.2, LLM-8.10</t>
+          <t>LLM-8.2, LLM-3.14</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2028,17 +2032,17 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>source_data</t>
+          <t>mcp_tools, agent</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Source data (RAG / knowledge graph)</t>
+          <t>MCP / tools (inside or outside); Agent</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -2049,7 +2053,7 @@
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>For the data your AI retrieves to answer questions, how are retrievals and changes to that data logged, showing who asked and what was returned, so that access to sensitive content through the AI can be traced? Who reviews these logs?</t>
+          <t>For your highest-criticality AI systems, how is each action the AI takes through tools or on your systems logged, with the credentials or identity it used and what it did, so that it can be traced back to the request and approval behind it? Who reviews these logs, and how long are they kept?</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2059,7 +2063,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.2, LLM-3.14</t>
+          <t>MCP-8.1, MCP-8.2, MCP-8.5, AGENT-8.1, AGENT-8.2, AGENT-8.5, AGENT-8.9</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2087,17 +2091,17 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>mcp_tools, agent</t>
+          <t>hosting</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>MCP / tools (inside or outside); Agent</t>
+          <t>Hosting</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -2108,7 +2112,7 @@
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>For your highest-criticality AI systems, how is each action the AI takes through tools or on your systems logged, with the credentials or identity it used and what it did, so that it can be traced back to the request and approval behind it? Who reviews these logs, and how long are they kept?</t>
+          <t>For your highest-criticality AI systems that you host, how are administrative actions, model registry changes, secret access and serving endpoint activity logged so that actions can be traced and accounted for? Who reviews them, and how often?</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -2118,7 +2122,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>MCP-8.1, MCP-8.2, MCP-8.5, AGENT-8.1, AGENT-8.2, AGENT-8.5, AGENT-8.9</t>
+          <t>LLM-8.2, LLM-8.1, LLM-8.9</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2136,48 +2140,52 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8</t>
+          <t>MANAGE 3.2</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Risks associated with transparency and accountability – as identified in the MAP function – are examined and documented.</t>
+          <t>Pre-trained models which are used for development are monitored as part of AI system regular monitoring and maintenance.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>hosting</t>
+          <t>model_building</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Model building</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>consumer, producer</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr"/>
+          <t>producer</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>built_on_existing_model</t>
+        </is>
+      </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>For the environment where you host AI models, how are administrative actions, model registry changes, secret access and serving endpoint activity logged so that actions can be traced and accounted for? Who reviews them, and how often?</t>
+          <t>For the pre-trained base models you build on, how are they tracked and monitored, for example for published vulnerabilities? Who owns this?</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>MEASURE 2.8 — suggested action 1</t>
+          <t>MANAGE 3.2 — suggested action 1, MANAGE 3.2 — suggested action 2</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>LLM-8.2, LLM-8.1, LLM-8.9</t>
+          <t>LLM-16.2, LLM-2.1</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2188,77 +2196,14 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>human</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>MANAGE 3.2</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Pre-trained models which are used for development are monitored as part of AI system regular monitoring and maintenance.</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>model_building</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Model building</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>producer</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>built_on_existing_model</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>For the pre-trained base models you build on, how are they tracked and monitored, for example for published vulnerabilities? Who owns this?</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>MANAGE 3.2 — suggested action 1, MANAGE 3.2 — suggested action 2</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>LLM-16.2, LLM-2.1</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>pass</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="inlineStr">
-        <is>
           <t>agent</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M31"/>
+  <autoFilter ref="A1:M30"/>
   <dataValidations count="1">
-    <dataValidation sqref="K2:K231" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K2:K230" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"pass,needs_human_review"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Evidence prompts in the AI banks (Step 6b run): 247 of 287 stored
Sonnet writers, Opus evaluators, one per part (foundation; areas MAP, MEASURE,
MANAGE). Stored: foundation 74 of 84, areas 173 of 203. The 40 that failed keep the
generic line; almost all asked for "the latest alert / incident / example" without
"if any". The writer prompt now says such events are always asked as "the latest one,
if any", so a rerun of Step 6b covers only those 40. Review sheets refreshed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LfWLLRUPBVgScvEVMJMnXw
</commit_message>
<xml_diff>
--- a/data/ai/authoring/questions_areas.xlsx
+++ b/data/ai/authoring/questions_areas.xlsx
@@ -566,7 +566,11 @@
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>The intended-purpose record for each customer-facing AI system (customer types, settings, applicable laws), its named owner, and the date of its last review.</t>
+        </is>
+      </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -626,7 +630,11 @@
           <t>LLM-3.2</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>The register of vendor products with AI features, showing per feature the data processed and its use, plus the most recent addition found and how it was found.</t>
+        </is>
+      </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -682,7 +690,11 @@
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>The written definition of a correct answer for each highest-criticality AI system (acceptance criteria or reference examples), its owner, and when it was last updated.</t>
+        </is>
+      </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -738,7 +750,11 @@
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>The roster or meeting record for the latest model build or tuning review, showing participants' roles, domains and user-experience backgrounds, and any bias or misuse concern they raised.</t>
+        </is>
+      </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -910,7 +926,11 @@
           <t>LLM-16.1</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>The requirements document for the latest model build or tuning (privacy, security, trustworthiness), showing who the requirements came from and the build decisions that trace to them.</t>
+        </is>
+      </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -966,7 +986,11 @@
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>The retrieval access requirements (who may see which content) for each highest-criticality AI system, the owner, and the permission configuration that implements them.</t>
+        </is>
+      </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1022,7 +1046,11 @@
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>The model design record stating its task and chosen method (built from scratch or tuned), the approval and approver, and the latest change to either.</t>
+        </is>
+      </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1082,7 +1110,11 @@
           <t>AGENT-1.1, AGENT-2.1</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>The agent specification for each highest-criticality AI system listing its tasks, tools and systems it uses, the record owner, and the last update date.</t>
+        </is>
+      </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1142,7 +1174,11 @@
           <t>LLM-14.1</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>The limitations document or user guidance for each highest-criticality AI system (known output limits, out-of-scope situations), where reviewers can find it, and the latest revision.</t>
+        </is>
+      </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1198,7 +1234,11 @@
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>A screenshot or text of the customer-facing notice about AI limits and possible errors, the screens where it appears, and its last change.</t>
+        </is>
+      </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1258,7 +1298,11 @@
           <t>LLM-15.1</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>The vendor AI documentation per feature (model provider, sub-processors, stated limits), the owner, and the date it was last refreshed.</t>
+        </is>
+      </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1314,7 +1358,11 @@
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>The model card or equivalent listing the model's limits and settings outside its intended use, its maintainer, and the latest version date.</t>
+        </is>
+      </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1374,7 +1422,11 @@
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>The release notes or model documentation sent with the latest model release to others, showing the limits and out-of-scope settings communicated, and the distribution channel, if any.</t>
+        </is>
+      </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1430,7 +1482,11 @@
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>The notice or documentation of topics the retrieval data does not cover, the place users see it in each highest-criticality AI system, and its last update.</t>
+        </is>
+      </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1490,7 +1546,11 @@
           <t>MCP-12.4, MCP-15.1, LLM-12.4</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>The diagram or list of external servers, networks and endpoints each highest-criticality AI system connects to, the data flowing to each, its owner, and the last review.</t>
+        </is>
+      </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1550,7 +1610,11 @@
           <t>LLM-3.2</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>The dataset documentation for the model's training, tuning, evaluation and test sets (sources, selection criteria, representativeness checks) for the latest model version.</t>
+        </is>
+      </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1606,7 +1670,11 @@
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>The test-data separation record for the latest evaluation (de-duplication or overlap check result, how test cases are held apart) and the name of the person who checked it.</t>
+        </is>
+      </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1666,7 +1734,11 @@
           <t>LLM-3.1</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>The source selection record for the retrieval content of each highest-criticality AI system (suitability, quality and trust checks per source), and the latest source added or removed.</t>
+        </is>
+      </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1722,7 +1794,11 @@
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>The latest benefit assessment for each highest-criticality AI system, such as a comparison of AI results against a person doing the task, with user input gathered and the owner.</t>
+        </is>
+      </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1778,7 +1854,11 @@
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Customer feedback or research records (surveys, interviews, usage analysis) on benefit and valued features for each customer-facing AI system, and the latest results.</t>
+        </is>
+      </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1834,7 +1914,11 @@
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>The build-versus-existing-model assessment for the latest model the organisation built or tuned, showing the benefits compared, the sign-off and its date.</t>
+        </is>
+      </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1890,7 +1974,11 @@
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>The latest findings on why staff use unapproved AI tools (survey, interview or usage-review notes), the approved alternatives assessed against them, and the follow-up owner.</t>
+        </is>
+      </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -1946,7 +2034,11 @@
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>The cost-of-error estimate for each highest-criticality AI system in internal decisions, with the past incidents or feedback it draws on, and where it is recorded.</t>
+        </is>
+      </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2002,7 +2094,11 @@
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>The likelihood and impact ratings (benefits and harms) for AI in internal decisions of each highest-criticality AI system, the reviewer, and the latest review date.</t>
+        </is>
+      </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2058,7 +2154,11 @@
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>The customer and business cost analysis of wrong, harmful or leaked answers for each customer-facing AI system, the reviewer, and its latest revision.</t>
+        </is>
+      </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2114,7 +2214,11 @@
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>The assessment of cost and affected groups from wrong, manipulated or biased answers for each highest-criticality AI system, where recorded, and the date.</t>
+        </is>
+      </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2170,7 +2274,11 @@
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>The impact analysis of hosting compromise, outage and cost abuse for each highest-criticality hosted AI system, compared with the stated risk tolerance, and the owner.</t>
+        </is>
+      </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2282,7 +2390,11 @@
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>The code-generation policy or standard listing where AI-generated code is allowed and prohibited (authentication, cryptography, regulated code), and the enforcement mechanism such as a repository rule.</t>
+        </is>
+      </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2338,7 +2450,11 @@
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>The scope definition for each customer-facing AI system (what it may answer or do, restrictions against public misuse), its reviewer, and the latest review date.</t>
+        </is>
+      </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2394,7 +2510,11 @@
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
-      <c r="K34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>The register of vendor AI features with the systems, data classes and uses each is limited to, and the setting or approval that enforces each limit.</t>
+        </is>
+      </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2454,7 +2574,11 @@
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
-      <c r="K35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>The release scope specification (users, products, regions) for the latest model release given to others, and the approval for any release outside it, if any.</t>
+        </is>
+      </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2570,7 +2694,11 @@
           <t>MCP-6.8, MCP-5.5</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>The tool scope list for each highest-criticality AI system (permitted reads, writes, actions and credentials per tool), compared to the use case need, with the approver and date.</t>
+        </is>
+      </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2630,7 +2758,11 @@
           <t>AGENT-6.8</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>The autonomy specification for each agent (permitted systems, actions, data, and actions never delegated), its location, and the latest change.</t>
+        </is>
+      </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2690,7 +2822,11 @@
           <t>LLM-14.1</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>The oversight procedure for each highest-criticality AI system (when to check, challenge or override output), the training attendance records for staff, and the latest update.</t>
+        </is>
+      </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2750,7 +2886,11 @@
           <t>LLM-16.1, LLM-16.8</t>
         </is>
       </c>
-      <c r="K40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>The code review policy for AI-generated code, plus a recent merge record or pull request showing the review and its approver.</t>
+        </is>
+      </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2806,7 +2946,11 @@
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
-      <c r="K41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>The guidance given to reviewers of AI-generated code on likely weaknesses and what not to rely on it for, where it is published, and its last update.</t>
+        </is>
+      </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2918,7 +3062,11 @@
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
-      <c r="K43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>The list of tool actions that need human confirmation (writes, deletes, payments, external sends) for each highest-criticality AI system, its location, owner, and last change.</t>
+        </is>
+      </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -2974,7 +3122,11 @@
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
-      <c r="K44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>The configuration or workflow showing that confirmation is enforced before high-impact tool actions run, a log extract of a recent confirmation with the confirming person, and the list of confirmers.</t>
+        </is>
+      </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3030,7 +3182,11 @@
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
-      <c r="K45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>The definition of which agent steps require human approval or review in each highest-criticality AI system, the reviewer roster, and a recent approval record.</t>
+        </is>
+      </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3086,7 +3242,11 @@
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
-      <c r="K46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>The training material and attendance records for agent action reviewers, and the latest oversight test (date, scenario, result) for each highest-criticality AI system.</t>
+        </is>
+      </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3146,7 +3306,11 @@
           <t>LLM-16.4, LLM-2.1</t>
         </is>
       </c>
-      <c r="K47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>The record of AI-suggested packages and libraries (name, source, check result for made-up names), its location, and the latest case where a non-existent package was caught, if any.</t>
+        </is>
+      </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3206,7 +3370,11 @@
           <t>LLM-15.1, LLM-15.4</t>
         </is>
       </c>
-      <c r="K48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>The vendor AI risk assessment for each vendor (model provider, data retention and training use, terms of service), its owner, and the latest reassessment date.</t>
+        </is>
+      </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3266,7 +3434,11 @@
           <t>LLM-15.5</t>
         </is>
       </c>
-      <c r="K49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>The security and resilience evaluation for each vendor AI (data separation from other customers, unavailability fallback), its latest date, and the repeat schedule.</t>
+        </is>
+      </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3326,7 +3498,11 @@
           <t>LLM-16.4, LLM-2.1</t>
         </is>
       </c>
-      <c r="K50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>The legal, licence and IP risk assessment of the base model or component used in the latest model build or tuning, and where the result is recorded.</t>
+        </is>
+      </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3386,7 +3562,11 @@
           <t>LLM-1.2, LLM-1.3, LLM-1.5, LLM-3.2</t>
         </is>
       </c>
-      <c r="K51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>The discovery list of unapproved AI tools, features, experiments and local models, the data each receives, the discovery method (such as network or expense review), the list owner, and last update.</t>
+        </is>
+      </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3446,7 +3626,11 @@
           <t>LLM-1.2, LLM-1.3, LLM-1.5</t>
         </is>
       </c>
-      <c r="K52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>The list of outside AI agents connecting to your systems, the discovery method (such as access log or API review), its owner, and the latest review date.</t>
+        </is>
+      </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3506,7 +3690,11 @@
           <t>LLM-3.2</t>
         </is>
       </c>
-      <c r="K53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>The review of provider terms on keeping or reusing prompts and files for each outside provider used by highest-criticality AI systems, where it is recorded, and the review date.</t>
+        </is>
+      </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3566,7 +3754,11 @@
           <t>LLM-3.2</t>
         </is>
       </c>
-      <c r="K54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>The register of third-party and licensed data used for training, tuning and testing (source, usage rights, licence risk), with its owner and the latest addition.</t>
+        </is>
+      </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3626,7 +3818,11 @@
           <t>LLM-2.1</t>
         </is>
       </c>
-      <c r="K55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>The decision record on weights and version ownership and the release licence, including infringement risk review notes, the decision maker, and the latest review date.</t>
+        </is>
+      </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3686,7 +3882,11 @@
           <t>LLM-3.2</t>
         </is>
       </c>
-      <c r="K56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>The rights record for third-party or external content feeding each highest-criticality AI system's retrieval data (licence or permission per source), its location, and the latest check.</t>
+        </is>
+      </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3746,7 +3946,11 @@
           <t>MCP-1.1, MCP-2.1, MCP-15.1</t>
         </is>
       </c>
-      <c r="K57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>The inventory of tools and MCP servers each highest-criticality AI system can call, including who runs each, its owner, and the date it was last reconciled with actual configuration.</t>
+        </is>
+      </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3806,7 +4010,11 @@
           <t>LLM-1.1, LLM-2.1</t>
         </is>
       </c>
-      <c r="K58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>The inventory of servers, GPUs, registries and serving software for each hosted highest-criticality AI system, with the mapped risks, its owner, and the last update.</t>
+        </is>
+      </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3866,7 +4074,11 @@
           <t>LLM-16.4, LLM-16.5</t>
         </is>
       </c>
-      <c r="K59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>The package check procedure and a recent result (existence, source and vulnerability check on AI-suggested packages), the approved source list, and the person responsible.</t>
+        </is>
+      </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3926,7 +4138,11 @@
           <t>LLM-15.4</t>
         </is>
       </c>
-      <c r="K60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>The control settings per vendor AI feature (training off, history retention off, permitted data classes), the document recording the decision, and the latest verification of the settings.</t>
+        </is>
+      </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -3986,7 +4202,11 @@
           <t>LLM-2.1, LLM-2.3</t>
         </is>
       </c>
-      <c r="K61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>The approved list of base models and components for building, the decision record behind it, its owner, and the latest addition or removal.</t>
+        </is>
+      </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4046,7 +4266,11 @@
           <t>LLM-2.5, LLM-9.2, LLM-9.4</t>
         </is>
       </c>
-      <c r="K62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>The configuration of controls limiting staff AI services, extensions and software (safelist, DNS or extension policy), the maintaining team, and the latest change.</t>
+        </is>
+      </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4106,7 +4330,11 @@
           <t>LLM-3.1</t>
         </is>
       </c>
-      <c r="K63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>The review record for third-party datasets and reused feedback or logs before they entered a training, tuning or test set (bias, privacy, poisoning checks), and the approver.</t>
+        </is>
+      </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4166,7 +4394,11 @@
           <t>LLM-3.3, LLM-3.7</t>
         </is>
       </c>
-      <c r="K64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>The retrieval access rules for each highest-criticality AI system (for example by content classification), a test showing a restricted item not returned, and the approver.</t>
+        </is>
+      </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4226,7 +4458,11 @@
           <t>MCP-6.1, MCP-2.5</t>
         </is>
       </c>
-      <c r="K65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>The approval records for tools and MCP servers in each highest-criticality AI system, the allowed-version list, and where these controls are documented.</t>
+        </is>
+      </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4286,7 +4522,11 @@
           <t>AGENT-2.1, AGENT-2.5, AGENT-2.6</t>
         </is>
       </c>
-      <c r="K66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>The component inventory for each agent (models, orchestration frameworks, libraries, executors) with approved versions, its owner, and the latest drift check.</t>
+        </is>
+      </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4346,7 +4586,11 @@
           <t>AGENT-16.4, AGENT-16.5</t>
         </is>
       </c>
-      <c r="K67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>The licence, IP and supply-chain review of models, frameworks and libraries behind each agent, with the reviewer, date, and any issue raised.</t>
+        </is>
+      </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4406,7 +4650,11 @@
           <t>LLM-2.5, LLM-2.6</t>
         </is>
       </c>
-      <c r="K68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>The review and approval records for third-party hosting material (base images, serving software, models, packages) with the scan result, the approver, and the latest approval.</t>
+        </is>
+      </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4462,7 +4710,11 @@
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr"/>
-      <c r="K69" s="2" t="inlineStr"/>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>The risk ratings (likelihood, severity, data sensitivity) for found unapproved AI use and outside agents, the prioritised list, and the person who decides order of handling.</t>
+        </is>
+      </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4522,7 +4774,11 @@
           <t>LLM-3.7, LLM-3.2</t>
         </is>
       </c>
-      <c r="K70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>The exposure assessment of prompts and files for each highest-criticality AI system, based on actual sent data (such as log or sample analysis), its owner, and the latest date.</t>
+        </is>
+      </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4582,7 +4838,11 @@
           <t>LLM-16.3</t>
         </is>
       </c>
-      <c r="K71" s="2" t="inlineStr"/>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>The latest red-team or test report on wrong or manipulated answers (including prompt injection) per highest-criticality AI system, the harm ratings, and the reviewer's sign-off.</t>
+        </is>
+      </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4642,7 +4902,11 @@
           <t>MCP-16.14, AGENT-16.14</t>
         </is>
       </c>
-      <c r="K72" s="2" t="inlineStr"/>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>The assessment of harm from AI actions on your systems (injected instructions, excess permissions, irreversible changes) per highest-criticality AI system, with its owner and date.</t>
+        </is>
+      </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4702,7 +4966,11 @@
           <t>LLM-17.8</t>
         </is>
       </c>
-      <c r="K73" s="2" t="inlineStr"/>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>The risk assessment of cost abuse and compromise of serving endpoints and GPUs for each hosted system, the past incidents drawn on, and how results set priorities.</t>
+        </is>
+      </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4814,7 +5082,11 @@
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr"/>
-      <c r="K75" s="2" t="inlineStr"/>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>The latest TEVV review record or sign-off for one top-criticality AI system, showing the reviewer's name, role and independence from the build team, the date, and the findings raised. Include the list of AI systems this review covers.</t>
+        </is>
+      </c>
       <c r="L75" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4870,7 +5142,11 @@
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr"/>
-      <c r="K76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>The TEVV documentation for one top-criticality AI system: the test sets, metrics and tools used for accuracy, consistency and bias, and the date they were last updated. Say which AI systems have this documentation and which do not.</t>
+        </is>
+      </c>
       <c r="L76" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4926,7 +5202,11 @@
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr"/>
-      <c r="K77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>A test plan or design note for one top-criticality AI system giving the rationale for the chosen test data and what each test is meant to measure, with the reviewer's approval and its date. Say which AI systems have such a note.</t>
+        </is>
+      </c>
       <c r="L77" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -4986,7 +5266,11 @@
           <t>LLM-3.2, LLM-11.2</t>
         </is>
       </c>
-      <c r="K78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>The version history or repository log for the evaluation and test sets, metric definitions and test tools of one critical model, showing version tags tied to model releases and the latest change. Say which models this covers.</t>
+        </is>
+      </c>
       <c r="L78" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5042,7 +5326,11 @@
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr"/>
-      <c r="K79" s="2" t="inlineStr"/>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>The most recent gap analysis comparing the people and situations in the test cases with those actually affected, for one top-criticality AI system, with the findings, the reviewer and any follow-up actions. Say which systems it covers.</t>
+        </is>
+      </c>
       <c r="L79" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5098,7 +5386,11 @@
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr"/>
-      <c r="K80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>The approval record and consent or data-protection check for the latest evaluation set drawn from people (user feedback, human-subject data), with the approver and the consent basis. If none is used, the rule that governs when one would be.</t>
+        </is>
+      </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5154,7 +5446,11 @@
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr"/>
-      <c r="K81" s="2" t="inlineStr"/>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>The latest performance test report for one top-criticality AI system showing realistic and messy inputs (real prompts, edge cases) alongside ideal ones, the results, and where they are stored. Say which systems and which deployment conditions it covers.</t>
+        </is>
+      </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5566,7 +5862,11 @@
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr"/>
-      <c r="K88" s="2" t="inlineStr"/>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>The model version monitoring or registry-comparison output for one critical model showing the deployed version against the approved one, the alert recipient, and the latest mismatch or change event, if any, with its review.</t>
+        </is>
+      </c>
       <c r="L88" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5686,7 +5986,11 @@
           <t>MCP-8.11, MCP-8.9</t>
         </is>
       </c>
-      <c r="K90" s="2" t="inlineStr"/>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>The tool and MCP server monitoring rules for one top-criticality AI system (unexpected calls, new capabilities on a known server, volume thresholds), the alert recipients, and a recent alert or review. Say which servers are covered.</t>
+        </is>
+      </c>
       <c r="L90" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5806,7 +6110,11 @@
           <t>LLM-13.2</t>
         </is>
       </c>
-      <c r="K92" s="2" t="inlineStr"/>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>The file integrity or configuration monitoring settings on the hosts for one critical model (model files, serving configuration), the alert recipients, and the latest alert or review record. Say which hosts are covered.</t>
+        </is>
+      </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5862,7 +6170,11 @@
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr"/>
-      <c r="K93" s="2" t="inlineStr"/>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>The pre-release validation report for one top-criticality AI system showing accuracy and consistency results, and the document stating the conditions and limits beyond which its answers cannot be trusted, with the approval date.</t>
+        </is>
+      </c>
       <c r="L93" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5922,7 +6234,11 @@
           <t>AGENT-16.13</t>
         </is>
       </c>
-      <c r="K94" s="2" t="inlineStr"/>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>The pre-release test results for one top-criticality agent under realistic tasks, and the document stating what the agent must not do on its own (autonomy limits, approvals needed), with its owner and approval date. Say which agents are covered.</t>
+        </is>
+      </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5978,7 +6294,11 @@
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr"/>
-      <c r="K95" s="2" t="inlineStr"/>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>The fail-safe test record for one top-criticality AI-supported internal process, showing the manual fallback or hand-off procedure, the scenarios tried (wrong, unavailable, out-of-limits output), the date of the last test and its result.</t>
+        </is>
+      </c>
       <c r="L95" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6038,7 +6358,11 @@
           <t>LLM-16.13</t>
         </is>
       </c>
-      <c r="K96" s="2" t="inlineStr"/>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>The latest test report showing a top-criticality AI system declining, flagging or handing over when outside its knowledge limits, with the test cases, results, date and who reviewed it. Say which systems are covered.</t>
+        </is>
+      </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6098,7 +6422,11 @@
           <t>LLM-16.13</t>
         </is>
       </c>
-      <c r="K97" s="2" t="inlineStr"/>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t>The latest abuse-resistance test report for one public-facing AI system (hostile and manipulative prompts), with the test cases, results, fixes made, date and who reviewed it. Say which customer-facing systems are covered.</t>
+        </is>
+      </c>
       <c r="L97" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6154,7 +6482,11 @@
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr"/>
-      <c r="K98" s="2" t="inlineStr"/>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t>The latest test record showing retrieval refusing restricted content when permission or classification checks fail or the data store misbehaves, for one top-criticality AI system, with the date, results and any fixes. Say which stores are covered.</t>
+        </is>
+      </c>
       <c r="L98" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6210,7 +6542,11 @@
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr"/>
-      <c r="K99" s="2" t="inlineStr"/>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t>The latest test record for one top-criticality AI system showing behaviour when a tool or MCP server errors, times out or returns unexpected output (stop, no retry loop, no partial changes), with the date, results and fixes.</t>
+        </is>
+      </c>
       <c r="L99" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6270,7 +6606,11 @@
           <t>AGENT-16.10, AGENT-17.9, AGENT-16.13</t>
         </is>
       </c>
-      <c r="K100" s="2" t="inlineStr"/>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>The latest stress test report for one top-criticality agent showing loop and runaway action-chain cases, the limits or kill switch that stopped them, the results, the date and who reviewed it. Say which agents are covered.</t>
+        </is>
+      </c>
       <c r="L100" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6330,7 +6670,11 @@
           <t>LLM-11.5</t>
         </is>
       </c>
-      <c r="K101" s="2" t="inlineStr"/>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>The latest recovery test record for the servers hosting one critical model, showing the restore of the model and configuration, the verification step, the date, the outcome, and the test schedule. Say which hosting environments are covered.</t>
+        </is>
+      </c>
       <c r="L101" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6390,7 +6734,11 @@
           <t>LLM-16.3</t>
         </is>
       </c>
-      <c r="K102" s="2" t="inlineStr"/>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t>The latest security test report for the AI coding assistant (non-existent or malicious package suggestions, poisoned context), with the test cases, results, date and follow-up actions. Say which assistants and teams are covered.</t>
+        </is>
+      </c>
       <c r="L102" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6450,7 +6798,11 @@
           <t>LLM-18.2, LLM-16.13, LLM-16.3</t>
         </is>
       </c>
-      <c r="K103" s="2" t="inlineStr"/>
+      <c r="K103" s="2" t="inlineStr">
+        <is>
+          <t>The latest prompt injection test report for one top-criticality AI system, covering user input and retrieved content, with the test cases, results, fixes, date and tester. Say which systems are covered.</t>
+        </is>
+      </c>
       <c r="L103" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6510,7 +6862,11 @@
           <t>LLM-13.3, MCP-13.10, AGENT-13.10</t>
         </is>
       </c>
-      <c r="K104" s="2" t="inlineStr"/>
+      <c r="K104" s="2" t="inlineStr">
+        <is>
+          <t>The latest test or exercise record for how your systems cope with outside AI agents, scrapers or MCP clients at machine speed (sign-in checks, rate limits, filtering), with the results and date. Say which services are covered.</t>
+        </is>
+      </c>
       <c r="L104" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6570,7 +6926,11 @@
           <t>LLM-3.1, LLM-3.3, LLM-6.8</t>
         </is>
       </c>
-      <c r="K105" s="2" t="inlineStr"/>
+      <c r="K105" s="2" t="inlineStr">
+        <is>
+          <t>The access control list and change log for the datasets used to build and evaluate one critical model, with integrity checks or hashes and the latest change review showing the reviewer. Say which models and datasets are covered.</t>
+        </is>
+      </c>
       <c r="L105" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6626,7 +6986,11 @@
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr"/>
-      <c r="K106" s="2" t="inlineStr"/>
+      <c r="K106" s="2" t="inlineStr">
+        <is>
+          <t>The latest security test report for one critical model covering theft, API extraction and version tampering, with the test cases, results, date and where it is stored. Say which models are covered.</t>
+        </is>
+      </c>
       <c r="L106" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6686,7 +7050,11 @@
           <t>LLM-3.3, LLM-3.12</t>
         </is>
       </c>
-      <c r="K107" s="2" t="inlineStr"/>
+      <c r="K107" s="2" t="inlineStr">
+        <is>
+          <t>The latest test report for one top-criticality AI system showing attempts to retrieve content a user should not reach, with the test users, results, fixes and date. Say which data stores are covered.</t>
+        </is>
+      </c>
       <c r="L107" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6746,7 +7114,11 @@
           <t>MCP-16.13</t>
         </is>
       </c>
-      <c r="K108" s="2" t="inlineStr"/>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>The latest security test report for the tools and MCP servers one top-criticality AI system can call (injection-driven tool calls, permission abuse), with the results, fixes and date. Say which servers are covered.</t>
+        </is>
+      </c>
       <c r="L108" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6806,7 +7178,11 @@
           <t>AGENT-16.13, AGENT-18.1, AGENT-18.5</t>
         </is>
       </c>
-      <c r="K109" s="2" t="inlineStr"/>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>The latest red-team report for one top-criticality agent with manipulated-input scenarios that trigger actions, the findings, fixes and retest, and the date. Say which agents have been red-teamed.</t>
+        </is>
+      </c>
       <c r="L109" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6866,7 +7242,11 @@
           <t>LLM-7.5, LLM-7.6</t>
         </is>
       </c>
-      <c r="K110" s="2" t="inlineStr"/>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t>The latest vulnerability scan or adversarial exercise report for the servers and exposed endpoints hosting one model, with the findings, owners and remediation status. Say which hosts are covered.</t>
+        </is>
+      </c>
       <c r="L110" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6926,7 +7306,11 @@
           <t>LLM-8.1, LLM-8.2, LLM-8.5, LLM-8.10</t>
         </is>
       </c>
-      <c r="K111" s="2" t="inlineStr"/>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t>A sample record for one high-impact decision or answer from a top-criticality AI system showing the AI output, the human review or override, and the output relied on, plus the log retention setting and the reviewer. Say which systems are covered.</t>
+        </is>
+      </c>
       <c r="L111" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -6986,7 +7370,11 @@
           <t>LLM-8.1, LLM-8.2, LLM-8.5</t>
         </is>
       </c>
-      <c r="K112" s="2" t="inlineStr"/>
+      <c r="K112" s="2" t="inlineStr">
+        <is>
+          <t>An extract of the AI code generation log (user, tool, prompt, generated code, merge link), the list of tools and teams it covers, who can read it, and the retention setting.</t>
+        </is>
+      </c>
       <c r="L112" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -7046,7 +7434,11 @@
           <t>LLM-8.12, LLM-8.2, LLM-8.1</t>
         </is>
       </c>
-      <c r="K113" s="2" t="inlineStr"/>
+      <c r="K113" s="2" t="inlineStr">
+        <is>
+          <t>The vendor's activity log or your own log extract showing what a vendor AI feature did with your data, the review schedule, and the latest review record. Say which vendor AI features are covered.</t>
+        </is>
+      </c>
       <c r="L113" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -7106,7 +7498,11 @@
           <t>LLM-8.1, LLM-8.2</t>
         </is>
       </c>
-      <c r="K114" s="2" t="inlineStr"/>
+      <c r="K114" s="2" t="inlineStr">
+        <is>
+          <t>An extract of the model build, tuning and release log (who, what, when) for one model, the list of models covered, and the latest review record with the reviewer.</t>
+        </is>
+      </c>
       <c r="L114" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -7166,7 +7562,11 @@
           <t>LLM-8.1, LLM-8.2, LLM-8.6, MCP-8.2</t>
         </is>
       </c>
-      <c r="K115" s="2" t="inlineStr"/>
+      <c r="K115" s="2" t="inlineStr">
+        <is>
+          <t>A log extract or report showing staff access to AI services and outside AI agents or tools calling your systems, including the identity recorded, the sources covered, and the latest review record.</t>
+        </is>
+      </c>
       <c r="L115" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -7226,7 +7626,11 @@
           <t>LLM-8.1, LLM-8.2, LLM-8.5, LLM-8.3</t>
         </is>
       </c>
-      <c r="K116" s="2" t="inlineStr"/>
+      <c r="K116" s="2" t="inlineStr">
+        <is>
+          <t>An extract of the prompt and response log for one top-criticality AI system showing sender, content and time, the access list for the logs, and the retention setting. Say which systems are covered.</t>
+        </is>
+      </c>
       <c r="L116" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -7346,7 +7750,11 @@
           <t>LLM-8.2, LLM-8.1</t>
         </is>
       </c>
-      <c r="K118" s="2" t="inlineStr"/>
+      <c r="K118" s="2" t="inlineStr">
+        <is>
+          <t>An extract of the change and access log for the training, tuning and evaluation data and the test harness, showing named individuals, plus the latest review record and who reviewed it. Say which datasets are covered.</t>
+        </is>
+      </c>
       <c r="L118" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -7406,7 +7814,11 @@
           <t>LLM-8.1, LLM-8.2, LLM-8.10</t>
         </is>
       </c>
-      <c r="K119" s="2" t="inlineStr"/>
+      <c r="K119" s="2" t="inlineStr">
+        <is>
+          <t>An extract of the access and change log for one model's weights, system prompts, configuration and version changes, tied to named people, plus the retention setting and latest review record.</t>
+        </is>
+      </c>
       <c r="L119" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -7466,7 +7878,11 @@
           <t>LLM-8.2, LLM-3.14</t>
         </is>
       </c>
-      <c r="K120" s="2" t="inlineStr"/>
+      <c r="K120" s="2" t="inlineStr">
+        <is>
+          <t>An extract of the retrieval and data-change log for one top-criticality AI system (requester, query, content returned, changes to the store), the latest review record, and the stores covered.</t>
+        </is>
+      </c>
       <c r="L120" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -7526,7 +7942,11 @@
           <t>MCP-8.1, MCP-8.2, MCP-8.5, AGENT-8.1, AGENT-8.2, AGENT-8.5, AGENT-8.9</t>
         </is>
       </c>
-      <c r="K121" s="2" t="inlineStr"/>
+      <c r="K121" s="2" t="inlineStr">
+        <is>
+          <t>An extract of the action log for one top-criticality AI system showing each tool or system action with the identity or credentials used, the originating request and the approval, plus the retention setting and latest review. Say which agents and servers are covered.</t>
+        </is>
+      </c>
       <c r="L121" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -7586,7 +8006,11 @@
           <t>LLM-8.2, LLM-8.1, LLM-8.9</t>
         </is>
       </c>
-      <c r="K122" s="2" t="inlineStr"/>
+      <c r="K122" s="2" t="inlineStr">
+        <is>
+          <t>A log extract of administrative actions, model registry changes, secret access and serving endpoint activity for one hosted AI system, the review frequency and latest review record. Say which hosted systems are covered.</t>
+        </is>
+      </c>
       <c r="L122" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -7642,7 +8066,11 @@
         </is>
       </c>
       <c r="J123" s="2" t="inlineStr"/>
-      <c r="K123" s="2" t="inlineStr"/>
+      <c r="K123" s="2" t="inlineStr">
+        <is>
+          <t>Screenshots or samples of how one top-criticality AI system presents answers (basis, confidence level, known limits), the design decision record saying who decided what context is shown, and the date. Say which systems are covered.</t>
+        </is>
+      </c>
       <c r="L123" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -7762,7 +8190,11 @@
           <t>LLM-3.13</t>
         </is>
       </c>
-      <c r="K125" s="2" t="inlineStr"/>
+      <c r="K125" s="2" t="inlineStr">
+        <is>
+          <t>The monitoring rules for personal or confidential data in answers from one public-facing AI system, the latest detected leak or review with its outcome, and the reviewer. Say which customer-facing systems are covered.</t>
+        </is>
+      </c>
       <c r="L125" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8002,7 +8434,11 @@
           <t>LLM-3.7, LLM-3.1</t>
         </is>
       </c>
-      <c r="K129" s="2" t="inlineStr"/>
+      <c r="K129" s="2" t="inlineStr">
+        <is>
+          <t>The privacy review or data minimisation record for one model's training and tuning data (discovery scan, removal or masking steps), and the document recording reuse of feedback or logs for tuning. Say which models are covered.</t>
+        </is>
+      </c>
       <c r="L129" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8062,7 +8498,11 @@
           <t>LLM-3.7, LLM-3.13</t>
         </is>
       </c>
-      <c r="K130" s="2" t="inlineStr"/>
+      <c r="K130" s="2" t="inlineStr">
+        <is>
+          <t>The classification or discovery scan report for the data store one top-criticality AI system retrieves from, showing personal and sensitive data found, the exposure assessment and the named owner. Say which stores are covered.</t>
+        </is>
+      </c>
       <c r="L130" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8122,7 +8562,11 @@
           <t>MCP-8.7, MCP-15.3</t>
         </is>
       </c>
-      <c r="K131" s="2" t="inlineStr"/>
+      <c r="K131" s="2" t="inlineStr">
+        <is>
+          <t>The privacy risk assessment for one top-criticality AI system's tool and MCP server use, showing what personal data goes to which servers or outside services, with the reviewer and date. Say which servers are covered.</t>
+        </is>
+      </c>
       <c r="L131" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8178,7 +8622,11 @@
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr"/>
-      <c r="K132" s="2" t="inlineStr"/>
+      <c r="K132" s="2" t="inlineStr">
+        <is>
+          <t>The privacy risk assessment for one top-criticality agent covering memory kept across sessions and data moved between systems, with retention settings, the named owner and date. Say which agents are covered.</t>
+        </is>
+      </c>
       <c r="L132" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8234,7 +8682,11 @@
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr"/>
-      <c r="K133" s="2" t="inlineStr"/>
+      <c r="K133" s="2" t="inlineStr">
+        <is>
+          <t>The latest bias test report for one top-criticality AI system comparing treatment of people or groups, with the method, groups compared, results, date and where it is stored. Say which systems are covered.</t>
+        </is>
+      </c>
       <c r="L133" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8290,7 +8742,11 @@
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr"/>
-      <c r="K134" s="2" t="inlineStr"/>
+      <c r="K134" s="2" t="inlineStr">
+        <is>
+          <t>The environmental impact assessment or compute and energy usage report for training and tuning runs of one critical model, with the method used, the latest figures and where it is recorded. Say which models are covered.</t>
+        </is>
+      </c>
       <c r="L134" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8346,7 +8802,11 @@
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr"/>
-      <c r="K135" s="2" t="inlineStr"/>
+      <c r="K135" s="2" t="inlineStr">
+        <is>
+          <t>The most recent review of the accuracy, consistency and bias tests for one top-criticality AI system, showing whether they catch known bad answers, the reviewer, the date, and the review schedule. Say which systems are covered.</t>
+        </is>
+      </c>
       <c r="L135" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8402,7 +8862,11 @@
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr"/>
-      <c r="K136" s="2" t="inlineStr"/>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>The latest review record for the evaluation set and test harness of one model, showing refresh dates, checks that the set has not leaked into training, the reviewer, and the review schedule.</t>
+        </is>
+      </c>
       <c r="L136" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8518,7 +8982,11 @@
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr"/>
-      <c r="K138" s="2" t="inlineStr"/>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t>The customer feedback or appeal channel for one customer-facing AI system (form, contact route, appeal procedure), the latest summary of counted and analysed reports, and the named owner. Say which systems are covered.</t>
+        </is>
+      </c>
       <c r="L138" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8694,7 +9162,11 @@
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr"/>
-      <c r="K141" s="2" t="inlineStr"/>
+      <c r="K141" s="2" t="inlineStr">
+        <is>
+          <t>The latest staff feedback survey results or override-rate report for one top-criticality internal AI system, showing over- or under-reliance measures, the reviewer and date. Say which systems are covered.</t>
+        </is>
+      </c>
       <c r="L141" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8750,7 +9222,11 @@
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr"/>
-      <c r="K142" s="2" t="inlineStr"/>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>The latest summary of user feedback (positive and negative) and override rates for one top-criticality AI system, with the review record and the named reviewer. Say which systems and user groups are covered.</t>
+        </is>
+      </c>
       <c r="L142" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8806,7 +9282,11 @@
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr"/>
-      <c r="K143" s="2" t="inlineStr"/>
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>The latest validation record from domain experts or users for one top-criticality AI system (sample answers checked, results, consistency), the names and roles of those involved, the date, and the schedule.</t>
+        </is>
+      </c>
       <c r="L143" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8862,7 +9342,11 @@
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr"/>
-      <c r="K144" s="2" t="inlineStr"/>
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>The baseline definition and the latest trend report for answer quality of one top-criticality AI system, showing improvements or declines over time, the dates compared, and where the results are stored. Say which systems are covered.</t>
+        </is>
+      </c>
       <c r="L144" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8922,7 +9406,11 @@
           <t>LLM-15.6</t>
         </is>
       </c>
-      <c r="K145" s="2" t="inlineStr"/>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>The register of vendor AI features that touch your data with each feature's keep/disable decision, risk rationale and named owner, plus the latest record where a vendor change (new feature or terms) was reviewed, and the feature's data settings.</t>
+        </is>
+      </c>
       <c r="L145" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8982,7 +9470,11 @@
           <t>LLM-16.8</t>
         </is>
       </c>
-      <c r="K146" s="2" t="inlineStr"/>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>The release approval record for the latest model version you built or tuned: the intended-purpose criteria, evaluation results against them, the go/no-go decision, approver and date. Say which models it covers and the release gate procedure.</t>
+        </is>
+      </c>
       <c r="L146" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9038,7 +9530,11 @@
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr"/>
-      <c r="K147" s="2" t="inlineStr"/>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>For each highest-criticality AI system, the latest evaluation report against its stated purpose and acceptance thresholds, the continue/stop decision with decision-maker and date, and the procedure that sets how often this is reviewed.</t>
+        </is>
+      </c>
       <c r="L147" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9094,7 +9590,11 @@
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr"/>
-      <c r="K148" s="2" t="inlineStr"/>
+      <c r="K148" s="2" t="inlineStr">
+        <is>
+          <t>For each highest-criticality agent, the latest review combining test and monitoring results (task success, errors, overrides), the decision on keeping or changing its autonomy level, the named decider and date, and the review schedule.</t>
+        </is>
+      </c>
       <c r="L148" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9150,7 +9650,11 @@
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr"/>
-      <c r="K149" s="2" t="inlineStr"/>
+      <c r="K149" s="2" t="inlineStr">
+        <is>
+          <t>The business rules, second-approval steps or output limits configured for each highest-criticality internal-decision AI system, the list of decisions they cover, the latest log or sample showing a blocked or escalated case, and who last confirmed them.</t>
+        </is>
+      </c>
       <c r="L149" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9210,7 +9714,11 @@
           <t>LLM-13.10, LLM-16.11</t>
         </is>
       </c>
-      <c r="K150" s="2" t="inlineStr"/>
+      <c r="K150" s="2" t="inlineStr">
+        <is>
+          <t>The guardrail configuration (output filters, throttling, action limits) for each highest-criticality AI system, the latest test or log extract showing a block firing, and the record of the last check that these controls still work.</t>
+        </is>
+      </c>
       <c r="L150" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9270,7 +9778,11 @@
           <t>LLM-3.1, LLM-3.13</t>
         </is>
       </c>
-      <c r="K151" s="2" t="inlineStr"/>
+      <c r="K151" s="2" t="inlineStr">
+        <is>
+          <t>The data-handling rule and the filter, redaction or DLP configuration applied to prompts for each highest-criticality AI system, a recent log extract of blocked or masked sensitive data, and the latest check of its effectiveness.</t>
+        </is>
+      </c>
       <c r="L151" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9330,7 +9842,11 @@
           <t>LLM-3.1, LLM-3.4, LLM-3.5</t>
         </is>
       </c>
-      <c r="K152" s="2" t="inlineStr"/>
+      <c r="K152" s="2" t="inlineStr">
+        <is>
+          <t>The data management procedure for training, tuning and test data covering quality checks, minimisation, retention schedule and deletion on request, the named owner, and the latest example of a deletion or quality check carried out, if any.</t>
+        </is>
+      </c>
       <c r="L152" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9450,7 +9966,11 @@
           <t>LLM-3.4, LLM-3.5</t>
         </is>
       </c>
-      <c r="K154" s="2" t="inlineStr"/>
+      <c r="K154" s="2" t="inlineStr">
+        <is>
+          <t>For each highest-criticality retrieval-based AI system, the source content inventory with owners and review dates, the retirement or refresh procedure, and the latest example of outdated material removed from the index.</t>
+        </is>
+      </c>
       <c r="L154" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9510,7 +10030,11 @@
           <t>MCP-5.2, MCP-6.7, MCP-6.8</t>
         </is>
       </c>
-      <c r="K155" s="2" t="inlineStr"/>
+      <c r="K155" s="2" t="inlineStr">
+        <is>
+          <t>The permission settings and credential configuration (scopes, expiry, rate limits) of each tool and MCP server the highest-criticality AI systems call, compared to user permissions, and the record of the latest review of them.</t>
+        </is>
+      </c>
       <c r="L155" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9630,7 +10154,11 @@
           <t>LLM-12.3, LLM-12.2</t>
         </is>
       </c>
-      <c r="K157" s="2" t="inlineStr"/>
+      <c r="K157" s="2" t="inlineStr">
+        <is>
+          <t>For each self-hosted highest-criticality AI system, the serving endpoint configuration (authentication gateway, network isolation rules, rate limits), the list of who can reach it, and the latest review or scan of this setup.</t>
+        </is>
+      </c>
       <c r="L157" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9690,7 +10218,11 @@
           <t>LLM-17.4, LLM-17.3</t>
         </is>
       </c>
-      <c r="K158" s="2" t="inlineStr"/>
+      <c r="K158" s="2" t="inlineStr">
+        <is>
+          <t>The procedure for responding to a decision based on wrong or misused AI output, with the named response lead, and the latest incident or exercise record showing how the decision was reversed, the AI's use corrected and lessons captured, if any.</t>
+        </is>
+      </c>
       <c r="L158" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9750,7 +10282,11 @@
           <t>LLM-17.4, LLM-17.3</t>
         </is>
       </c>
-      <c r="K159" s="2" t="inlineStr"/>
+      <c r="K159" s="2" t="inlineStr">
+        <is>
+          <t>The response procedure for a secret leaked into a prompt or a bad dependency introduced by an AI coding tool (rotation, removal, dependency review), and the latest incident or exercise record with lead, actions and date, if any.</t>
+        </is>
+      </c>
       <c r="L159" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9810,7 +10346,11 @@
           <t>LLM-17.4</t>
         </is>
       </c>
-      <c r="K160" s="2" t="inlineStr"/>
+      <c r="K160" s="2" t="inlineStr">
+        <is>
+          <t>The response procedure for customer-reported AI problems and newly found risks in each highest-criticality customer-facing AI system, the named owner, and the latest case record from report to closure, if any.</t>
+        </is>
+      </c>
       <c r="L160" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9930,7 +10470,11 @@
           <t>LLM-17.4, LLM-17.8</t>
         </is>
       </c>
-      <c r="K162" s="2" t="inlineStr"/>
+      <c r="K162" s="2" t="inlineStr">
+        <is>
+          <t>The response and rebuild procedure for a problem in a released model, naming the lead, the steps to retrain, restore or withdraw the version, and the latest incident or exercise record showing the rebuild, if any.</t>
+        </is>
+      </c>
       <c r="L162" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10050,7 +10594,11 @@
           <t>LLM-17.4, LLM-17.3</t>
         </is>
       </c>
-      <c r="K164" s="2" t="inlineStr"/>
+      <c r="K164" s="2" t="inlineStr">
+        <is>
+          <t>The procedure for sensitive data found sent to a model or provider (containment, provider deletion request, recovery), the named lead, and the latest incident or exercise record, with the provider's response, if any.</t>
+        </is>
+      </c>
       <c r="L164" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10110,7 +10658,11 @@
           <t>LLM-17.4</t>
         </is>
       </c>
-      <c r="K165" s="2" t="inlineStr"/>
+      <c r="K165" s="2" t="inlineStr">
+        <is>
+          <t>The response procedure for newly found output problems (injection route, bias, drift) in each highest-criticality AI system, the named lead, and the latest incident record showing detection, fix, re-test and closure, if any.</t>
+        </is>
+      </c>
       <c r="L165" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10170,7 +10722,11 @@
           <t>LLM-17.4, LLM-11.1, LLM-11.5</t>
         </is>
       </c>
-      <c r="K166" s="2" t="inlineStr"/>
+      <c r="K166" s="2" t="inlineStr">
+        <is>
+          <t>The procedure for restoring a clean verified copy of training, tuning and evaluation data and test cases after poisoning or tampering, the backup and integrity-check records, and the latest restore test or incident record, if any.</t>
+        </is>
+      </c>
       <c r="L166" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10230,7 +10786,11 @@
           <t>LLM-17.4, LLM-17.3</t>
         </is>
       </c>
-      <c r="K167" s="2" t="inlineStr"/>
+      <c r="K167" s="2" t="inlineStr">
+        <is>
+          <t>The response procedure for a stolen, leaked or tampered model or configuration (revocation, rollback, rebuild), the named lead, and the latest incident or exercise record, if any.</t>
+        </is>
+      </c>
       <c r="L167" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10290,7 +10850,11 @@
           <t>LLM-17.4</t>
         </is>
       </c>
-      <c r="K168" s="2" t="inlineStr"/>
+      <c r="K168" s="2" t="inlineStr">
+        <is>
+          <t>The runbook for putting a poisoned or leaked retrieval store right (removal of content, re-indexing, access review), the named runner, and the latest incident or exercise record covering each highest-criticality retrieval system, if any.</t>
+        </is>
+      </c>
       <c r="L168" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10350,7 +10914,11 @@
           <t>MCP-17.4, MCP-17.3</t>
         </is>
       </c>
-      <c r="K169" s="2" t="inlineStr"/>
+      <c r="K169" s="2" t="inlineStr">
+        <is>
+          <t>The incident procedure for tool or MCP server incidents (misused credential, injected call, compromised server) covering credential rotation and server isolation, the named lead, and the latest incident or exercise record, if any.</t>
+        </is>
+      </c>
       <c r="L169" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10410,7 +10978,11 @@
           <t>AGENT-17.4, AGENT-17.5</t>
         </is>
       </c>
-      <c r="K170" s="2" t="inlineStr"/>
+      <c r="K170" s="2" t="inlineStr">
+        <is>
+          <t>The agent incident runbook including how the agent's changes are listed and reversed, the named lead, the agent's action log used for it, and the latest incident or exercise record showing a rollback, if any.</t>
+        </is>
+      </c>
       <c r="L170" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10470,7 +11042,11 @@
           <t>LLM-17.4, LLM-11.1</t>
         </is>
       </c>
-      <c r="K171" s="2" t="inlineStr"/>
+      <c r="K171" s="2" t="inlineStr">
+        <is>
+          <t>The recovery procedure for a compromised, failed or abused self-hosted AI endpoint, backup and restore settings with the latest restore test, the named lead, and the latest incident or exercise record, if any.</t>
+        </is>
+      </c>
       <c r="L171" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10530,7 +11106,11 @@
           <t>LLM-17.9</t>
         </is>
       </c>
-      <c r="K172" s="2" t="inlineStr"/>
+      <c r="K172" s="2" t="inlineStr">
+        <is>
+          <t>For each highest-criticality AI system, the documented bypass or switch-off procedure and any trigger thresholds, the list of people authorised to use it, and the latest test or actual use of the switch-off with date and result.</t>
+        </is>
+      </c>
       <c r="L172" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10590,7 +11170,11 @@
           <t>LLM-17.9, LLM-17.4</t>
         </is>
       </c>
-      <c r="K173" s="2" t="inlineStr"/>
+      <c r="K173" s="2" t="inlineStr">
+        <is>
+          <t>The procedure and settings to disable an AI coding assistant or revoke its access, the named decider, the secret-leak or bad-package trigger criteria, and the latest test or actual use of the switch-off, if any.</t>
+        </is>
+      </c>
       <c r="L173" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10650,7 +11234,11 @@
           <t>LLM-15.7, LLM-17.9</t>
         </is>
       </c>
-      <c r="K174" s="2" t="inlineStr"/>
+      <c r="K174" s="2" t="inlineStr">
+        <is>
+          <t>For each vendor AI feature on your data, the admin setting or contract clause allowing it to be turned off or access revoked, the named person who can do so, and the latest instance or test of disabling a feature, if any.</t>
+        </is>
+      </c>
       <c r="L174" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10774,7 +11362,11 @@
           <t>LLM-2.3, LLM-6.2, MCP-1.2, AGENT-1.2</t>
         </is>
       </c>
-      <c r="K176" s="2" t="inlineStr"/>
+      <c r="K176" s="2" t="inlineStr">
+        <is>
+          <t>The blocking and access revocation procedure for unapproved AI tools and outside agents or MCP clients (network, identity and gateway controls), the named authorised people, and the latest case where access was blocked and revoked, if any.</t>
+        </is>
+      </c>
       <c r="L176" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10834,7 +11426,11 @@
           <t>LLM-17.9</t>
         </is>
       </c>
-      <c r="K177" s="2" t="inlineStr"/>
+      <c r="K177" s="2" t="inlineStr">
+        <is>
+          <t>For each highest-criticality AI system, the control that stops input going to a model or provider (egress block, key disablement), the named decider, and the latest test or actual use with date and result.</t>
+        </is>
+      </c>
       <c r="L177" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10894,7 +11490,11 @@
           <t>LLM-11.1, LLM-6.2</t>
         </is>
       </c>
-      <c r="K178" s="2" t="inlineStr"/>
+      <c r="K178" s="2" t="inlineStr">
+        <is>
+          <t>The rollback procedure to a trusted model version, the model registry or version history showing approved versions, the access revocation steps, and the latest rollback test or actual withdrawal record, if any.</t>
+        </is>
+      </c>
       <c r="L178" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10954,7 +11554,11 @@
           <t>LLM-17.9</t>
         </is>
       </c>
-      <c r="K179" s="2" t="inlineStr"/>
+      <c r="K179" s="2" t="inlineStr">
+        <is>
+          <t>For each highest-criticality retrieval-based system, the steps and settings to disconnect a source or the whole store from retrieval, the named decider, and the latest test or actual disconnection record, if any.</t>
+        </is>
+      </c>
       <c r="L179" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11074,7 +11678,11 @@
           <t>AGENT-6.2, AGENT-17.9</t>
         </is>
       </c>
-      <c r="K181" s="2" t="inlineStr"/>
+      <c r="K181" s="2" t="inlineStr">
+        <is>
+          <t>For each highest-criticality agent, the stop or kill-switch setting, the access revocation steps for its identity, the list of people authorised to use them, and the latest test or actual use with date and outcome.</t>
+        </is>
+      </c>
       <c r="L181" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11134,7 +11742,11 @@
           <t>LLM-17.9</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr"/>
+      <c r="K182" s="2" t="inlineStr">
+        <is>
+          <t>For each self-hosted AI endpoint, the procedure and settings to disable or isolate it and revoke its API keys, the people authorised to do so, any cost or abuse alert thresholds, and the latest test or actual use.</t>
+        </is>
+      </c>
       <c r="L182" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11194,7 +11806,11 @@
           <t>LLM-15.6</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr"/>
+      <c r="K183" s="2" t="inlineStr">
+        <is>
+          <t>The vendor AI change-monitoring record (new AI features, model provider changes, terms updates) with the date of the latest review, the check that agreed data controls still apply, the named owner, and the vendor list it covers.</t>
+        </is>
+      </c>
       <c r="L183" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11250,7 +11866,11 @@
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr"/>
-      <c r="K184" s="2" t="inlineStr"/>
+      <c r="K184" s="2" t="inlineStr">
+        <is>
+          <t>For each highest-criticality retrieval-based system, the list of third-party and external content sources feeding the index, the schedule and record of their latest re-review, any risk found, and the named owner.</t>
+        </is>
+      </c>
       <c r="L184" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11310,7 +11930,11 @@
           <t>MCP-15.6</t>
         </is>
       </c>
-      <c r="K185" s="2" t="inlineStr"/>
+      <c r="K185" s="2" t="inlineStr">
+        <is>
+          <t>The inventory of outside MCP servers and tool suppliers for each highest-criticality AI system, the change-monitoring record (new versions, changed permissions) with its latest date, and where the risk controls applied to each are documented.</t>
+        </is>
+      </c>
       <c r="L185" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11366,7 +11990,11 @@
         </is>
       </c>
       <c r="J186" s="2" t="inlineStr"/>
-      <c r="K186" s="2" t="inlineStr"/>
+      <c r="K186" s="2" t="inlineStr">
+        <is>
+          <t>The list of third-party hosting providers (cloud, GPU, model registry) used by each highest-criticality AI system, their latest risk review or assurance report, the issues found, and the reviewer.</t>
+        </is>
+      </c>
       <c r="L186" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11430,7 +12058,11 @@
           <t>LLM-16.2, LLM-2.1</t>
         </is>
       </c>
-      <c r="K187" s="2" t="inlineStr"/>
+      <c r="K187" s="2" t="inlineStr">
+        <is>
+          <t>The inventory of pre-trained base models you build on with source, version and owner, the vulnerability or advisory monitoring method and its latest review record, and any action taken on a finding, if any.</t>
+        </is>
+      </c>
       <c r="L187" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11486,7 +12118,11 @@
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr"/>
-      <c r="K188" s="2" t="inlineStr"/>
+      <c r="K188" s="2" t="inlineStr">
+        <is>
+          <t>For each highest-criticality customer-facing AI application, the channel for customer feedback, appeals and human-override requests, a recent log extract of items received and their outcomes, and the named reviewer and review frequency.</t>
+        </is>
+      </c>
       <c r="L188" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11542,7 +12178,11 @@
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr"/>
-      <c r="K189" s="2" t="inlineStr"/>
+      <c r="K189" s="2" t="inlineStr">
+        <is>
+          <t>The post-go-live re-test plan for each highest-criticality AI system (accuracy, bias, security, red teaming), its frequency, the latest test report with findings and actions, and the date of the last run.</t>
+        </is>
+      </c>
       <c r="L189" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11662,7 +12302,11 @@
           <t>MCP-15.7, AGENT-16.1</t>
         </is>
       </c>
-      <c r="K191" s="2" t="inlineStr"/>
+      <c r="K191" s="2" t="inlineStr">
+        <is>
+          <t>The change approval records for the latest change to tools, permissions or configuration (including removals) of each highest-criticality AI system, the approver, the change procedure, and the post-change check.</t>
+        </is>
+      </c>
       <c r="L191" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11722,7 +12366,11 @@
           <t>LLM-7.2</t>
         </is>
       </c>
-      <c r="K192" s="2" t="inlineStr"/>
+      <c r="K192" s="2" t="inlineStr">
+        <is>
+          <t>The change procedure for hosting stack updates (servers, GPU drivers, serving software), the post-update behaviour test results for the latest update to each highest-criticality AI system, and the rollout approval with approver and date.</t>
+        </is>
+      </c>
       <c r="L192" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11778,7 +12426,11 @@
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr"/>
-      <c r="K193" s="2" t="inlineStr"/>
+      <c r="K193" s="2" t="inlineStr">
+        <is>
+          <t>For each highest-criticality customer-facing AI application, the log of customer feedback with decisions on what to act on and who decided, the improvement measures set, and the latest release note showing a measured result.</t>
+        </is>
+      </c>
       <c r="L193" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11898,7 +12550,11 @@
         </is>
       </c>
       <c r="J195" s="2" t="inlineStr"/>
-      <c r="K195" s="2" t="inlineStr"/>
+      <c r="K195" s="2" t="inlineStr">
+        <is>
+          <t>The communication to recipients of the latest released model version (release notes, change summary, feedback channel), the log of feedback collected, and the procedure that sets how recipients are engaged before a release, if any.</t>
+        </is>
+      </c>
       <c r="L195" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11958,7 +12614,11 @@
           <t>LLM-18.3</t>
         </is>
       </c>
-      <c r="K196" s="2" t="inlineStr"/>
+      <c r="K196" s="2" t="inlineStr">
+        <is>
+          <t>For the latest wrong, biased or inconsistent answer found in each highest-criticality AI system, the fix record (prompt, data, model or rule change), the before/after re-test results showing improvement, and the sign-off with name and date.</t>
+        </is>
+      </c>
       <c r="L196" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -12018,7 +12678,11 @@
           <t>LLM-17.3, LLM-17.8, MCP-17.8, AGENT-17.3, AGENT-17.8</t>
         </is>
       </c>
-      <c r="K197" s="2" t="inlineStr"/>
+      <c r="K197" s="2" t="inlineStr">
+        <is>
+          <t>The AI error and incident register or ticket category for the highest-criticality AI systems, the latest recorded entry with cause analysis and reviewer, and the reporting procedure that covers the areas in scope, such as agents, tools and code generation.</t>
+        </is>
+      </c>
       <c r="L197" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -12074,7 +12738,11 @@
         </is>
       </c>
       <c r="J198" s="2" t="inlineStr"/>
-      <c r="K198" s="2" t="inlineStr"/>
+      <c r="K198" s="2" t="inlineStr">
+        <is>
+          <t>The procedure and decision rule for telling people affected by wrong or harmful AI results or unexpected actions, the named decider, and the latest notification sent or drafted, if any, covering the AI systems in scope.</t>
+        </is>
+      </c>
       <c r="L198" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -12134,7 +12802,11 @@
           <t>LLM-17.2, LLM-17.3</t>
         </is>
       </c>
-      <c r="K199" s="2" t="inlineStr"/>
+      <c r="K199" s="2" t="inlineStr">
+        <is>
+          <t>The route by which vendor AI problems reach you (vendor contact, notification clause in the contract or DPA), the latest vendor-reported issue recorded in your incident log, and the named person who followed it up, if any.</t>
+        </is>
+      </c>
       <c r="L199" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -12194,7 +12866,11 @@
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr"/>
-      <c r="K200" s="2" t="inlineStr"/>
+      <c r="K200" s="2" t="inlineStr">
+        <is>
+          <t>The notification procedure for recipients of a released model with error or incident, the named decider, the recipient contact list, and the latest notice sent, if any.</t>
+        </is>
+      </c>
       <c r="L200" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -12250,7 +12926,11 @@
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr"/>
-      <c r="K201" s="2" t="inlineStr"/>
+      <c r="K201" s="2" t="inlineStr">
+        <is>
+          <t>The change log or model registry history for the most critical models showing each change to the model or setup, the reason, the approver and date, and where the log is kept and who can edit it.</t>
+        </is>
+      </c>
       <c r="L201" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -12310,7 +12990,11 @@
           <t>LLM-17.3, LLM-17.8</t>
         </is>
       </c>
-      <c r="K202" s="2" t="inlineStr"/>
+      <c r="K202" s="2" t="inlineStr">
+        <is>
+          <t>The record of incidents and near-misses from unapproved AI use or outside agents reaching your systems, the latest entry showing who was told and the post-incident review, and the procedure for recording and communicating them, if any.</t>
+        </is>
+      </c>
       <c r="L202" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -12366,7 +13050,11 @@
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr"/>
-      <c r="K203" s="2" t="inlineStr"/>
+      <c r="K203" s="2" t="inlineStr">
+        <is>
+          <t>The notification procedure for exposed sensitive data sent to an AI, the decision record on who must be told (affected people, providers, regulators) with the decider, and the latest notification or exercise record, if any.</t>
+        </is>
+      </c>
       <c r="L203" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -12426,7 +13114,11 @@
           <t>LLM-17.3, LLM-17.8</t>
         </is>
       </c>
-      <c r="K204" s="2" t="inlineStr"/>
+      <c r="K204" s="2" t="inlineStr">
+        <is>
+          <t>For infrastructure hosting the most critical AI models, the incident log entries for compromise, outage or cost abuse, the communication sent to those affected, and the latest post-incident review with its lead, if any.</t>
+        </is>
+      </c>
       <c r="L204" s="2" t="inlineStr">
         <is>
           <t>pass</t>

</xml_diff>

<commit_message>
Evidence prompts re-run with the fixed writer prompt: 271 of 287 stored
The 40 questions without one were re-run: foundation 3 of 10 and areas 21 of 30
stored. 16 keep the generic line (their evidence implies a formal structure the org
may not have), which the engagement reviewer sharpens. Review sheets refreshed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LfWLLRUPBVgScvEVMJMnXw
</commit_message>
<xml_diff>
--- a/data/ai/authoring/questions_areas.xlsx
+++ b/data/ai/authoring/questions_areas.xlsx
@@ -2334,7 +2334,11 @@
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>The scope document or system card for each highest-criticality internal AI system listing permitted and out-of-bounds decisions and workflows, plus the approval record of the latest scope change, if any.</t>
+        </is>
+      </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5026,7 +5030,11 @@
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr"/>
-      <c r="K74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>The customer feedback channel for each highest-criticality customer-facing AI system (form, button or contact route), the reviewer roster, and the latest triage record showing action taken on a reported answer, if any.</t>
+        </is>
+      </c>
       <c r="L74" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5510,7 +5518,11 @@
           <t>LLM-8.11</t>
         </is>
       </c>
-      <c r="K82" s="2" t="inlineStr"/>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>The monitoring rules and alert routing for public-facing AI systems (abuse patterns, unusual answers), the named alert recipients, and an extract from the latest monitoring review or alert, if any.</t>
+        </is>
+      </c>
       <c r="L82" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5570,7 +5582,11 @@
           <t>LLM-15.6, LLM-8.12</t>
         </is>
       </c>
-      <c r="K83" s="2" t="inlineStr"/>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>The vendor AI change-monitoring procedure (release notes feeds, provider logs, model version checks), the vendor feature settings reviewed, and the latest follow-up record of an unannounced change, if any.</t>
+        </is>
+      </c>
       <c r="L83" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5630,7 +5646,11 @@
           <t>LLM-8.6, LLM-8.12, LLM-1.5</t>
         </is>
       </c>
-      <c r="K84" s="2" t="inlineStr"/>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>The detection configuration for unapproved AI use (DNS, network or provider telemetry rules), the alert routing, and the latest review or alert record, if any, covering the whole organisation.</t>
+        </is>
+      </c>
       <c r="L84" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5686,7 +5706,11 @@
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr"/>
-      <c r="K85" s="2" t="inlineStr"/>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>The detection rules or dashboards for external AI agents or clients reaching your systems (sign-in, API and traffic patterns), the alert recipients, and the latest alert and its follow-up, if any.</t>
+        </is>
+      </c>
       <c r="L85" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5806,7 +5830,11 @@
           <t>LLM-8.11</t>
         </is>
       </c>
-      <c r="K87" s="2" t="inlineStr"/>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>The API usage monitoring rules for models behind critical AI systems (rate and repetition thresholds), a log extract showing flagged usage, if any, and the record of who reviewed it.</t>
+        </is>
+      </c>
       <c r="L87" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5926,7 +5954,11 @@
           <t>LLM-8.11</t>
         </is>
       </c>
-      <c r="K89" s="2" t="inlineStr"/>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>The monitoring configuration for the retrieval data behind each highest-criticality AI system (content change or integrity checks), the alert routing, and the latest finding and notification record, if any.</t>
+        </is>
+      </c>
       <c r="L89" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8130,7 +8162,11 @@
           <t>LLM-3.13, LLM-3.14</t>
         </is>
       </c>
-      <c r="K124" s="2" t="inlineStr"/>
+      <c r="K124" s="2" t="inlineStr">
+        <is>
+          <t>The secret-detection setting or data loss prevention rule applied to prompts in code assistants, the teams and tools it covers, and the latest detection and follow-up record, if any.</t>
+        </is>
+      </c>
       <c r="L124" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8254,7 +8290,11 @@
           <t>LLM-3.13, LLM-3.14</t>
         </is>
       </c>
-      <c r="K126" s="2" t="inlineStr"/>
+      <c r="K126" s="2" t="inlineStr">
+        <is>
+          <t>The data loss prevention policy or rule set covering traffic to unapproved AI tools, the data types and users it covers, and the latest alert with its follow-up record, if any.</t>
+        </is>
+      </c>
       <c r="L126" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8314,7 +8354,11 @@
           <t>LLM-3.13, LLM-3.14</t>
         </is>
       </c>
-      <c r="K127" s="2" t="inlineStr"/>
+      <c r="K127" s="2" t="inlineStr">
+        <is>
+          <t>The monitoring and alert configuration for personal or sensitive data in prompts and uploaded files for each highest-criticality AI system, the responder roster, and the latest alert and response, if any.</t>
+        </is>
+      </c>
       <c r="L127" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8374,7 +8418,11 @@
           <t>LLM-8.11</t>
         </is>
       </c>
-      <c r="K128" s="2" t="inlineStr"/>
+      <c r="K128" s="2" t="inlineStr">
+        <is>
+          <t>The input monitoring report for each highest-criticality AI system (volumes, file types, unexpected input) compared with the pre-launch test profile, the alert threshold settings, and the latest deviation alert, if any.</t>
+        </is>
+      </c>
       <c r="L128" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -8926,7 +8974,11 @@
           <t>LLM-17.3</t>
         </is>
       </c>
-      <c r="K137" s="2" t="inlineStr"/>
+      <c r="K137" s="2" t="inlineStr">
+        <is>
+          <t>The staff channel for reporting or challenging AI output in internal processes (form, ticket queue or contact route), the reviewers, and the latest analysis report or trend summary of submitted reports, if any.</t>
+        </is>
+      </c>
       <c r="L137" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9046,7 +9098,11 @@
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr"/>
-      <c r="K139" s="2" t="inlineStr"/>
+      <c r="K139" s="2" t="inlineStr">
+        <is>
+          <t>The problem-reporting route published with each released model (contact, issue tracker or model card section), and the latest report, if any, with the resulting change to building or tuning.</t>
+        </is>
+      </c>
       <c r="L139" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -9106,7 +9162,11 @@
           <t>AGENT-17.3</t>
         </is>
       </c>
-      <c r="K140" s="2" t="inlineStr"/>
+      <c r="K140" s="2" t="inlineStr">
+        <is>
+          <t>The channel for reporting agent misbehaviour (form, ticket type or contact route), who receives it, and the latest agent evaluation record that used such reports, if any.</t>
+        </is>
+      </c>
       <c r="L140" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10094,7 +10154,11 @@
           <t>AGENT-6.8, AGENT-6.1, AGENT-2.7</t>
         </is>
       </c>
-      <c r="K156" s="2" t="inlineStr"/>
+      <c r="K156" s="2" t="inlineStr">
+        <is>
+          <t>The permission and identity settings for each highest-criticality agent (least-privilege roles, approval gates for irreversible steps, rate and cost caps), and the latest review record of those limits.</t>
+        </is>
+      </c>
       <c r="L156" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10410,7 +10474,11 @@
           <t>LLM-17.4, LLM-17.9</t>
         </is>
       </c>
-      <c r="K161" s="2" t="inlineStr"/>
+      <c r="K161" s="2" t="inlineStr">
+        <is>
+          <t>The response procedure for new risks in vendor AI features (changed data practice, vendor-side leak) with the named lead, vendor contact terms or DPA clauses, and the latest response record, if any.</t>
+        </is>
+      </c>
       <c r="L161" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -10534,7 +10602,11 @@
           <t>LLM-17.3, LLM-17.4, LLM-14.6</t>
         </is>
       </c>
-      <c r="K163" s="2" t="inlineStr"/>
+      <c r="K163" s="2" t="inlineStr">
+        <is>
+          <t>The incident response and staff reporting procedure for data leaving through unapproved AI tools or outside agents misusing access, the named reporting contact, and the latest such incident record, if any.</t>
+        </is>
+      </c>
       <c r="L163" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -11302,7 +11374,11 @@
           <t>LLM-17.9</t>
         </is>
       </c>
-      <c r="K175" s="2" t="inlineStr"/>
+      <c r="K175" s="2" t="inlineStr">
+        <is>
+          <t>The withdrawal or supersession procedure for released model versions, including how recipients are notified, the named responsible owner, and the latest withdrawal or recipient notice, if any.</t>
+        </is>
+      </c>
       <c r="L175" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -12242,7 +12318,11 @@
           <t>LLM-3.5</t>
         </is>
       </c>
-      <c r="K190" s="2" t="inlineStr"/>
+      <c r="K190" s="2" t="inlineStr">
+        <is>
+          <t>The deletion and correction request procedure showing how it reaches retrieval data and its index for each highest-criticality AI system, and the latest request log entry showing completion, if any.</t>
+        </is>
+      </c>
       <c r="L190" s="2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -12490,7 +12570,11 @@
           <t>LLM-4.1</t>
         </is>
       </c>
-      <c r="K194" s="2" t="inlineStr"/>
+      <c r="K194" s="2" t="inlineStr">
+        <is>
+          <t>The change and release approval records for models behind critical AI systems (build or tuning changes, new versions), the named approvers, and the latest approved release with its review evidence.</t>
+        </is>
+      </c>
       <c r="L194" s="2" t="inlineStr">
         <is>
           <t>pass</t>

</xml_diff>